<commit_message>
cierre(EXT-0): sellos de indice_formulas.md y trazabilidad.csv firmados sobre a1b4417 y SHA en el tracker — 1978 passed, 8 skipped (PyMuPDF sí · ventana Tk no)
Los seis IDs que EXT-0 cierra o deja parciales (EXT-N-04, EXT-G-03, PC-24,
PC-25, PC-29, PC-30) citan a1b4417 en la columna Commit / PR; los sellos de
los dos generados con SHA llevan ese mismo árbol. Sin cambio de contenido.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T7KJ97oW5uszpJ92mtPkVF
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -16136,7 +16136,7 @@
       </c>
       <c r="L245" s="6" t="inlineStr">
         <is>
-          <t>SHA_EXT0</t>
+          <t>a1b4417 — EXT-0 (2026-09-20); el cierre con los sellos es el commit siguiente</t>
         </is>
       </c>
     </row>
@@ -17068,7 +17068,7 @@
       </c>
       <c r="L261" s="6" t="inlineStr">
         <is>
-          <t>SHA_EXT0</t>
+          <t>a1b4417 — EXT-0 (2026-09-20); el cierre con los sellos es el commit siguiente</t>
         </is>
       </c>
     </row>
@@ -18464,7 +18464,7 @@
       </c>
       <c r="L285" s="6" t="inlineStr">
         <is>
-          <t>SHA_EXT0</t>
+          <t>a1b4417 — EXT-0 (2026-09-20); el cierre con los sellos es el commit siguiente</t>
         </is>
       </c>
     </row>
@@ -18526,7 +18526,7 @@
       </c>
       <c r="L286" s="6" t="inlineStr">
         <is>
-          <t>SHA_EXT0</t>
+          <t>a1b4417 — EXT-0 (2026-09-20); el cierre con los sellos es el commit siguiente</t>
         </is>
       </c>
     </row>
@@ -18762,7 +18762,7 @@
       </c>
       <c r="L290" s="6" t="inlineStr">
         <is>
-          <t>SHA_EXT0</t>
+          <t>a1b4417 — EXT-0 (2026-09-20); el cierre con los sellos es el commit siguiente</t>
         </is>
       </c>
     </row>
@@ -18824,7 +18824,7 @@
       </c>
       <c r="L291" s="6" t="inlineStr">
         <is>
-          <t>SHA_EXT0</t>
+          <t>a1b4417 — EXT-0 (2026-09-20); el cierre con los sellos es el commit siguiente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cierre(EXT-1): sellos de indice_formulas.md y trazabilidad.csv firmados sobre 9195e8d y SHA en el tracker — 2070 passed, 8 skipped (PyMuPDF sí · ventana Tk no)
Medido sobre origin/main en 9195e8d. Sin PyMuPDF: 2035 passed, 41 skipped
medidos antes de los dos tests de regresion del auditor adversarial (2037
derivado). Este commit solo añade los sellos y el SHA en la hoja Hallazgos.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkjN14s6Z7vHyYGB16XDMS
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -15904,7 +15904,7 @@
       </c>
       <c r="L241" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-1) — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. M2._exigir_sin_repetidos (adyacente, no adyacente y casi-duplicado 5e-10 dentro de TOL_UMBRAL_NORMATIVO) + MD._exigir_progreso (guardia de progreso, DatoInvalidoError sobre el criterio de la progresión, nunca bucle). API por valor y orden declarado intactos.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. M2._exigir_sin_repetidos (adyacente, no adyacente y casi-duplicado 5e-10 dentro de TOL_UMBRAL_NORMATIVO) + MD._exigir_progreso (guardia de progreso, DatoInvalidoError sobre el criterio de la progresión, nunca bucle). API por valor y orden declarado intactos.</t>
         </is>
       </c>
     </row>
@@ -16666,7 +16666,7 @@
       </c>
       <c r="L254" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-1) — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. Validación cerrada: M4._validar_ke (real, finito, `not ke &gt;= 0`) en perdida_carga y en la rama numérica de ke_declarado; declaracion.Procedencia.valor_de_la_celda + difiere_de_la_celda; declarar_desde_tabla exige nota si valor ≠ celda; M11 imprime «DIFIERE de la celda (0.5)». La FORMA (C5-02, clave de fila) queda en EXT-6: ver decisiones_diferidas.md. AUDITOR ADVERSARIAL (EXT-1): refutó la primera versión de la guardia de celda (rechazaba la CLAVE de fila de ke_entrada_cajon declarada por la GUI); corregido en la misma sesión (la celda sólo se cita para valores numéricos) con test de regresión.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. Validación cerrada: M4._validar_ke (real, finito, `not ke &gt;= 0`) en perdida_carga y en la rama numérica de ke_declarado; declaracion.Procedencia.valor_de_la_celda + difiere_de_la_celda; declarar_desde_tabla exige nota si valor ≠ celda; M11 imprime «DIFIERE de la celda (0.5)». La FORMA (C5-02, clave de fila) queda en EXT-6: ver decisiones_diferidas.md. AUDITOR ADVERSARIAL (EXT-1): refutó la primera versión de la guardia de celda (rechazaba la CLAVE de fila de ke_entrada_cajon declarada por la GUI); corregido en la misma sesión (la celda sólo se cita para valores numéricos) con test de regresión.</t>
         </is>
       </c>
     </row>
@@ -16728,7 +16728,7 @@
       </c>
       <c r="L255" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-1) — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. M2._espesor_valido: un validador para las dos ramas (Real y no bool, finito, `not t &gt; 0`, `return float(t)`), orden Pendiente → Faltante material → Faltante fila → Inválido conservado. Parametrizado -0.1, 0, True, -0.0, inf, nan, '0.1'.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. M2._espesor_valido: un validador para las dos ramas (Real y no bool, finito, `not t &gt; 0`, `return float(t)`), orden Pendiente → Faltante material → Faltante fila → Inválido conservado. Parametrizado -0.1, 0, True, -0.0, inf, nan, '0.1'.</t>
         </is>
       </c>
     </row>
@@ -16790,7 +16790,7 @@
       </c>
       <c r="L256" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-1) — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. establecer_valor_dinamico y escribir_valor_en_archivo rechazan un criterio de resolución Derivada con ValueError («se deriva de &lt;de&gt;; edite sus entradas»); cubre pestaña 2, --declarar y declaracion.declarar_valor. Docstring «DE CUALQUIER CRITERIO» y test «mismo rasero» actualizados.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. establecer_valor_dinamico y escribir_valor_en_archivo rechazan un criterio de resolución Derivada con ValueError («se deriva de &lt;de&gt;; edite sus entradas»); cubre pestaña 2, --declarar y declaracion.declarar_valor. Docstring «DE CUALQUIER CRITERIO» y test «mismo rasero» actualizados.</t>
         </is>
       </c>
     </row>
@@ -16852,7 +16852,7 @@
       </c>
       <c r="L257" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-1) — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. Sensibilidad estructurada {campo: (min, max)} evaluada por criterios_adoptados._verificar_dict; 'seccion_receptor' migrado de prosa a dict. Rechaza dict mal formado, claves desconocidas/faltantes, no-real por campo y fuera de rango por campo.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. Sensibilidad estructurada {campo: (min, max)} evaluada por criterios_adoptados._verificar_dict; 'seccion_receptor' migrado de prosa a dict. Rechaza dict mal formado, claves desconocidas/faltantes, no-real por campo y fuera de rango por campo.</t>
         </is>
       </c>
     </row>
@@ -16914,7 +16914,7 @@
       </c>
       <c r="L258" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-1) — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. M1._exigir_forma_del_mapa: Mapping exterior, filas ∈ CategoriaTR, campos ∈ {R, n}, reales finitos no bool; errata o clave desconocida → DatoInvalidoError con la ruta. Ya no se ignora en silencio.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. M1._exigir_forma_del_mapa: Mapping exterior, filas ∈ CategoriaTR, campos ∈ {R, n}, reales finitos no bool; errata o clave desconocida → DatoInvalidoError con la ruta. Ya no se ignora en silencio.</t>
         </is>
       </c>
     </row>
@@ -17154,7 +17154,7 @@
       </c>
       <c r="L262" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-1) — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. _verificar_sensibilidad exige len == 2 y orden del par bajo rango numérico; modelos.Material.__post_init__ con `not n_min &lt;= n_max` → DatoInvalidoError; M2._par_de_manning convierte la forma mala del par en DatoInvalidoError (un escalar ya no tumba la corrida). Auditor adversarial: Material.__post_init__ admite el (None, None) documentado de n_manning_hdpe (era TypeError latente); test añadido.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. _verificar_sensibilidad exige len == 2 y orden del par bajo rango numérico; modelos.Material.__post_init__ con `not n_min &lt;= n_max` → DatoInvalidoError; M2._par_de_manning convierte la forma mala del par en DatoInvalidoError (un escalar ya no tumba la corrida). Auditor adversarial: Material.__post_init__ admite el (None, None) documentado de n_manning_hdpe (era TypeError latente); test añadido.</t>
         </is>
       </c>
     </row>
@@ -17216,7 +17216,7 @@
       </c>
       <c r="L263" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-1) — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. 'ke_entrada' con ventana (0.2, 0.9) derivada de KE_HDS5_C2; 'v_max_tmc' y 'v_max_hdpe' con ventana (V_MIN, 4.572). perdida_carga valida el signo. La línea base cambia sólo en la fila «Sensibilidad declarada» de esas tres fichas.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. 'ke_entrada' con ventana (0.2, 0.9) derivada de KE_HDS5_C2; 'v_max_tmc' y 'v_max_hdpe' con ventana (V_MIN, 4.572). perdida_carga valida el signo. La línea base cambia sólo en la fila «Sensibilidad declarada» de esas tres fichas.</t>
         </is>
       </c>
     </row>
@@ -17394,7 +17394,7 @@
       </c>
       <c r="L266" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-1) — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. M3._validar_parametros y M4._validar_positivo en forma MAT-D13 (`not x &gt; 0`); control_salida valida `not TW &gt;= 0` y guardia de finitud a la salida (LimiteNumericoError nombrando el par L, TW). test_seccion_rectangular actualizado: el NaN se detiene en la puerta, el inf llega a la guardia de tirante_critico.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. M3._validar_parametros y M4._validar_positivo en forma MAT-D13 (`not x &gt; 0`); control_salida valida `not TW &gt;= 0` y guardia de finitud a la salida (LimiteNumericoError nombrando el par L, TW). test_seccion_rectangular actualizado: el NaN se detiene en la puerta, el inf llega a la guardia de tirante_critico.</t>
         </is>
       </c>
     </row>
@@ -18740,7 +18740,7 @@
       </c>
       <c r="L289" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-1) — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. MD.disenar_punto acumula los DatoFaltanteError y relanza el primero (con campo) cuando TODOS los candidatos faltan; el caso mixto sigue igual.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. MD.disenar_punto acumula los DatoFaltanteError y relanza el primero (con campo) cuando TODOS los candidatos faltan; el caso mixto sigue igual.</t>
         </is>
       </c>
     </row>
@@ -18984,7 +18984,7 @@
       </c>
       <c r="L293" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-1) — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. Guardia de salida en M7.factor_esviaje con umbral NOMBRADO (tolerancias.COS_ESVIAJE_MIN = (π/2)·ε/TOL_UMBRAL_NORMATIVO ≈ 3.5e-7; LimiteNumericoError para θ &gt; 89.99998°). NO corta 89.9° (10 313 m): ese umbral es un valor de proyecto sin fuente en normas/ y MAT-O18 ya decidió que sería un criterio [A]; ficha PC-32 en decisiones_diferidas.md Parte XVII. test_M7 MAT-O18 reescrito.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. Guardia de salida en M7.factor_esviaje con umbral NOMBRADO (tolerancias.COS_ESVIAJE_MIN = (π/2)·ε/TOL_UMBRAL_NORMATIVO ≈ 3.5e-7; LimiteNumericoError para θ &gt; 89.99998°). NO corta 89.9° (10 313 m): ese umbral es un valor de proyecto sin fuente en normas/ y MAT-O18 ya decidió que sería un criterio [A]; ficha PC-32 en decisiones_diferidas.md Parte XVII. test_M7 MAT-O18 reescrito.</t>
         </is>
       </c>
     </row>
@@ -19046,7 +19046,7 @@
       </c>
       <c r="L294" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-1) — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. cli._numero_externo excluye bool antes de float().</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. cli._numero_externo excluye bool antes de float().</t>
         </is>
       </c>
     </row>
@@ -19108,7 +19108,7 @@
       </c>
       <c r="L295" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-1) — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. cli.declarar_criterios rechaza la tupla que no viene escrita con paréntesis (`0,5`); `(0.010, 0.013)` sigue declarable.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. cli.declarar_criterios rechaza la tupla que no viene escrita con paréntesis (`0,5`); `(0.010, 0.013)` sigue declarable.</t>
         </is>
       </c>
     </row>
@@ -19170,7 +19170,7 @@
       </c>
       <c r="L296" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-1) — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. cli.main valida la plantilla antes de correr (_exigir_plantilla_valida: existe, pide marcadores y sólo del contrato) y arma la memoria antes de escribir el JSON; FileNotFoundError/ValueError/ErrorProyecto salen con código 2 y sin salida a medias.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. cli.main valida la plantilla antes de correr (_exigir_plantilla_valida: existe, pide marcadores y sólo del contrato) y arma la memoria antes de escribir el JSON; FileNotFoundError/ValueError/ErrorProyecto salen con código 2 y sin salida a medias.</t>
         </is>
       </c>
     </row>
@@ -19654,7 +19654,7 @@
       </c>
       <c r="L304" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-1) — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. EXT-1 cerró la mitad de validación (ventana, guardia del consumidor, procedencia veraz) y DIFIERE la migración de forma a EXT-6; ficha C5-02 actualizada en decisiones_diferidas.md.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. EXT-1 cerró la mitad de validación (ventana, guardia del consumidor, procedencia veraz) y DIFIERE la migración de forma a EXT-6; ficha C5-02 actualizada en decisiones_diferidas.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cierre(EXT-2): sellos de indice_formulas.md y trazabilidad.csv firmados sobre 929da05 y SHA en el tracker — 2089 passed, 8 skipped (PyMuPDF sí · ventana Tk no)
Par medido sobre un checkout limpio de origin/main (929da05).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015vdorMGpRtYhMikBd72qtU
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -16318,7 +16318,7 @@
       </c>
       <c r="L248" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-2) (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext2_multicelda_transicion.py (escritos en rojo con xfail strict y liberados al corregir). Reparto Q/N DENTRO de M4 (`M4.caudal_por_celda`, invocada por `resolver_control` en los dos caminos, `normal` inyectado o resuelto); `ResultadoHidraulico.Q_celda_m3s` y `numero_celdas` con default (Q sigue siendo el total: sus tres lectores lo imprimen como caudal del punto); `PasoDeMemoria` del reparto colgado de F3.CELDAS (emitido por M4 solo para el marco, antes de Manning); F4.MANNING y F4.YC_RECT sustituyen el Q de la celda; cita `HDS5_3ED.5.4.3#REPARTO` (PDF 151) verificada y añadida a las citas de F3.CELDAS; `MD._caudal_por_barril` es alias de la función de M4. Test espía: las tres piezas de M4 reciben 3.0 y nunca 9.0; HW_salida 1.045982117 m, control de salida. V6 NO se cambia (sigue `celdas == 1`): ficha EXT-2-01 en decisiones_diferidas.md.</t>
+          <t>929da05 — EXT-2 (2026-09-20), PR #32; el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext2_multicelda_transicion.py (escritos en rojo con xfail strict y liberados al corregir). Reparto Q/N DENTRO de M4 (`M4.caudal_por_celda`, invocada por `resolver_control` en los dos caminos, `normal` inyectado o resuelto); `ResultadoHidraulico.Q_celda_m3s` y `numero_celdas` con default (Q sigue siendo el total: sus tres lectores lo imprimen como caudal del punto); `PasoDeMemoria` del reparto colgado de F3.CELDAS (emitido por M4 solo para el marco, antes de Manning); F4.MANNING y F4.YC_RECT sustituyen el Q de la celda; cita `HDS5_3ED.5.4.3#REPARTO` (PDF 151) verificada y añadida a las citas de F3.CELDAS; `MD._caudal_por_barril` es alias de la función de M4. Test espía: las tres piezas de M4 reciben 3.0 y nunca 9.0; HW_salida 1.045982117 m, control de salida. V6 NO se cambia (sigue `celdas == 1`): ficha EXT-2-01 en decisiones_diferidas.md.</t>
         </is>
       </c>
     </row>
@@ -16380,7 +16380,7 @@
       </c>
       <c r="L249" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-2) (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext2_multicelda_transicion.py (escritos en rojo con xfail strict y liberados al corregir). `control_entrada`: Q_lo = 3.5·A_llena·√D/Ku y, solo bajo Forma 1, H_c_lo = tirante_critico(Q_lo).H_c en el extremo inferior; `ControlEntrada.transicion` (`modelos.TransicionEntrada`: Q_lo, H_c_lo, HW_lo, HW_hi, peso) y F4.CONTROL sustituye los cuatro; dorado CP5T_PUNTO_MEDIO_TRANSICION = 1.107921425 m calculado a mano en casos_patron; linealidad (segundas diferencias &lt; 1e-12) y continuidad en 3.5/4.0; justificación de `metodo_transicion_hds5` precisada. Línea base: A-01 −0.306 mm de HW_entrada (1.0423077 → 1.0420015 m) en informe_perfil_ancho.json y las tres memorias HTML.</t>
+          <t>929da05 — EXT-2 (2026-09-20), PR #32; el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext2_multicelda_transicion.py (escritos en rojo con xfail strict y liberados al corregir). `control_entrada`: Q_lo = 3.5·A_llena·√D/Ku y, solo bajo Forma 1, H_c_lo = tirante_critico(Q_lo).H_c en el extremo inferior; `ControlEntrada.transicion` (`modelos.TransicionEntrada`: Q_lo, H_c_lo, HW_lo, HW_hi, peso) y F4.CONTROL sustituye los cuatro; dorado CP5T_PUNTO_MEDIO_TRANSICION = 1.107921425 m calculado a mano en casos_patron; linealidad (segundas diferencias &lt; 1e-12) y continuidad en 3.5/4.0; justificación de `metodo_transicion_hds5` precisada. Línea base: A-01 −0.306 mm de HW_entrada (1.0423077 → 1.0420015 m) en informe_perfil_ancho.json y las tres memorias HTML.</t>
         </is>
       </c>
     </row>
@@ -17464,7 +17464,7 @@
       </c>
       <c r="L267" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-2) (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext2_multicelda_transicion.py (escritos en rojo con xfail strict y liberados al corregir). `M3.tirante_normal` compara Q con Q_lleno = (k_n/n)·A_llena·R_lleno^(2/3)·S^(1/2) (radio hidráulico de la sección llena, en las dos formas) y devuelve None si `not Q &lt; Q_lleno` (forma MAT-D13). Marco 2.00×1.50, Q = 8.0 → None (antes y/H = 0.864); Q_lleno = 7.70 m³/s. La circular no se mueve (el bracket ya ponía el mismo techo salvo el borde exacto).</t>
+          <t>929da05 — EXT-2 (2026-09-20), PR #32; el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext2_multicelda_transicion.py (escritos en rojo con xfail strict y liberados al corregir). `M3.tirante_normal` compara Q con Q_lleno = (k_n/n)·A_llena·R_lleno^(2/3)·S^(1/2) (radio hidráulico de la sección llena, en las dos formas) y devuelve None si `not Q &lt; Q_lleno` (forma MAT-D13). Marco 2.00×1.50, Q = 8.0 → None (antes y/H = 0.864); Q_lleno = 7.70 m³/s. La circular no se mueve (el bracket ya ponía el mismo techo salvo el borde exacto).</t>
         </is>
       </c>
     </row>
@@ -18164,7 +18164,7 @@
       </c>
       <c r="L279" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-2) (2026-09-20): línea base regenerada y ENSANCHADA. entradas_ampliadas.json declara TW_m = 1.00 m &gt; D = 0.90 m para B-01 (salida ahogada: h_o = TW, HW 0.36 → 0.82 m, control de salida; V1/V2 siguen [OK] sobre y_n: el caso de EXT-M-01 queda congelado y visible para EXT-3); punto_cajon.py declara n_celdas_cajon = 3 y pasa por el reparto de M4 (mutación «Q total a M4» ahora mueve memoria_punto_cajon.html). Lo que se movió, archivo por archivo, está en el README de la línea base (sección EXT-2).</t>
+          <t>929da05 — EXT-2 (2026-09-20), PR #32: línea base regenerada y ENSANCHADA. entradas_ampliadas.json declara TW_m = 1.00 m &gt; D = 0.90 m para B-01 (salida ahogada: h_o = TW, HW 0.36 → 0.82 m, control de salida; V1/V2 siguen [OK] sobre y_n: el caso de EXT-M-01 queda congelado y visible para EXT-3); punto_cajon.py declara n_celdas_cajon = 3 y pasa por el reparto de M4 (mutación «Q total a M4» ahora mueve memoria_punto_cajon.html). Lo que se movió, archivo por archivo, está en el README de la línea base (sección EXT-2).</t>
         </is>
       </c>
     </row>
@@ -18226,7 +18226,7 @@
       </c>
       <c r="L280" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-2) (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext2_multicelda_transicion.py (escritos en rojo con xfail strict y liberados al corregir). `test_la_interpolacion_reproduce_la_recta_entre_los_dos_extremos` reescrito con H_c(Q_lo) y con la afirmación de que el extremo móvil ya NO es el usado; tests de punto medio (media exacta de los extremos) y de linealidad en test_ext2_multicelda_transicion.py.</t>
+          <t>929da05 — EXT-2 (2026-09-20), PR #32; el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext2_multicelda_transicion.py (escritos en rojo con xfail strict y liberados al corregir). `test_la_interpolacion_reproduce_la_recta_entre_los_dos_extremos` reescrito con H_c(Q_lo) y con la afirmación de que el extremo móvil ya NO es el usado; tests de punto medio (media exacta de los extremos) y de linealidad en test_ext2_multicelda_transicion.py.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cierre(EXT-3): sellos de indice_formulas.md y trazabilidad.csv firmados sobre 43b2531 y SHA en el tracker — 2123 passed, 4 skipped (PyMuPDF sí · ventana Tk sí)
Las cuatro configuraciones medidas sobre origin/main en 43b2531 (collected
2127 = 2097 + 30): sí·sí 2123/4, sí·no 2119/8, no·sí 2090/37, no·no
2086/41. La columna Tk se midió instalando python3-tk en el contenedor y las
dos sin PyMuPDF desinstalándolo y reinstalándolo. Tabla de cuatro entornos y
párrafo de EXT-3 en CLAUDE.md; SHA 43b2531 en las filas EXT-M-01, EXT-M-02,
PC-04, PC-27, SIS-B-18 y NOR-HDS-05 del tracker.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011aDpvWqQ8M6NqR8iCmtdYG
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -4325,7 +4325,7 @@
       </c>
       <c r="L41" s="6" t="inlineStr">
         <is>
-          <t>4141fd5 — S19 — RAZON PRECISADA, sin cambio de codigo. Verificado hoy: las dos condiciones evaluables lo siguen siendo (H_O_HW_SOBRE_D_MIN y H_O_HW_SOBRE_D_CAUTELA, calculadas en control_salida e impresas en la memoria del punto) y la tercera --- que el barril fluya lleno en la mayor parte de su longitud --- sigue transcrita y DECLARADA como no evaluable en H_O_CONDICION_APLICACION, con M4 diciendolo en el punto de uso. QUE FALTA: el procedimiento de barril parcialmente lleno del Cap. III del HDS-5. Es implementar un metodo hidraulico: NO se cierra en F5. Ficha en docs/decisiones_diferidas.md. || S19d — SHA AÑADIDO, y la nota de arriba se lee bien: sin cambio de CODIGO, no sin commit. La razon precisada SI esta versionada --- es la ficha de este ID en la Parte III de docs/decisiones_diferidas.md, que nace en 4141fd5 (verificado: `git show 4141fd5:docs/decisiones_diferidas.md` ya trae las cuatro fichas NOR). Se corrige la celda y NO el verificador: relajar la exigencia de SHA para toda nota que diga «sin cambio de codigo» seria un guardian que se pone verde sobre una FRASE en vez de sobre el hecho, que es el modo de fallo de FACTOR_MURO_TABLA. || 183415b + 9902b3c — I1/I1b — EVALUADO LO QUE LA FICHA DEJABA POR EVALUAR: el Cap. III del HDS-5 3a ed. SI da el procedimiento de barril parcialmente lleno en forma transcribible, y el paquete de implementacion completo (prosa en 3.12/PDF 94 con la Ec. 3.7; umbrales de 3.24/PDF 106; Secc. 3.5 PDF 116-120; que implementar en M4 y por que M5 no cambia; dorados solo con corrida externa citable, conflicto #7) quedo ESCRITO en el bloque que precede a H_O_CONDICION_APLICACION, sin implementar: toca M4.control_salida, motor validado — es sesion propia con plan mode. Ficha de decisiones_diferidas actualizada. Veredicto regla 3 (auditor adversarial I1b): NO CIERRA y no pretende; el paquete es honesto y no contradice Conflictos. Sigue Cerrado parcial. || EXT-0 — REABIERTO con argumento nuevo (EXT-M-02, PC-27, PC-25): el «Cerrado parcial» descansaba en que HW/D &lt; 0.75 bajo control de salida fuera un AVISO; el punto se acepta con h_o_fuera_de_rango=True (sin lector fuera de M11) mientras el PasoDeMemoria del mismo punto imprime NO_CUMPLE (SIS-A-07). La v8 §4.3 decide ahora «método no evaluable» por vía Bloqueo, diferible en perfil y no en expediente, nunca cumple=False (subir D sólo baja HW/D, 0.589 → 0.526). Además el paquete I1 decía «M5 no cambia» y EXT-M-01 lo refuta (V1/V2 salen del régimen del barril bajo TW ahogante). La frase elidida de la pág. 3.24 está completa desde EXT-0 (v8 y H_O_CONDICION_TEXTO). Sesiones: EXT-3 (bloqueo, régimen) y E-A (perfil por paso directo). Ficha de decisiones_diferidas.md actualizada. || EXT-3 (2026-09-20) — CERRADO PARCIAL, con el argumento de EXT-0 resuelto: HW/D &lt; 0.75 bajo control de salida ya NO es un aviso sino `MetodoNoEvaluableError` por vía Bloqueo (diferible en perfil, no en expediente), F4.HO dice DIFERIDO y no NO_CUMPLE, y la compuerta lee el mismo campo (SIS-A-07). V1/V2 salen del régimen del barril (EXT-M-01). Lo ÚNICO que sigue abierto es la tercera condición —que el barril fluya lleno en la mayor parte de su longitud— y con ella el perfil por paso directo (EXT-3b / E-A), con el paquete I1 de H_O_CONDICION_APLICACION intacto.</t>
+          <t>4141fd5 — S19 — RAZON PRECISADA, sin cambio de codigo. Verificado hoy: las dos condiciones evaluables lo siguen siendo (H_O_HW_SOBRE_D_MIN y H_O_HW_SOBRE_D_CAUTELA, calculadas en control_salida e impresas en la memoria del punto) y la tercera --- que el barril fluya lleno en la mayor parte de su longitud --- sigue transcrita y DECLARADA como no evaluable en H_O_CONDICION_APLICACION, con M4 diciendolo en el punto de uso. QUE FALTA: el procedimiento de barril parcialmente lleno del Cap. III del HDS-5. Es implementar un metodo hidraulico: NO se cierra en F5. Ficha en docs/decisiones_diferidas.md. || S19d — SHA AÑADIDO, y la nota de arriba se lee bien: sin cambio de CODIGO, no sin commit. La razon precisada SI esta versionada --- es la ficha de este ID en la Parte III de docs/decisiones_diferidas.md, que nace en 4141fd5 (verificado: `git show 4141fd5:docs/decisiones_diferidas.md` ya trae las cuatro fichas NOR). Se corrige la celda y NO el verificador: relajar la exigencia de SHA para toda nota que diga «sin cambio de codigo» seria un guardian que se pone verde sobre una FRASE en vez de sobre el hecho, que es el modo de fallo de FACTOR_MURO_TABLA. || 183415b + 9902b3c — I1/I1b — EVALUADO LO QUE LA FICHA DEJABA POR EVALUAR: el Cap. III del HDS-5 3a ed. SI da el procedimiento de barril parcialmente lleno en forma transcribible, y el paquete de implementacion completo (prosa en 3.12/PDF 94 con la Ec. 3.7; umbrales de 3.24/PDF 106; Secc. 3.5 PDF 116-120; que implementar en M4 y por que M5 no cambia; dorados solo con corrida externa citable, conflicto #7) quedo ESCRITO en el bloque que precede a H_O_CONDICION_APLICACION, sin implementar: toca M4.control_salida, motor validado — es sesion propia con plan mode. Ficha de decisiones_diferidas actualizada. Veredicto regla 3 (auditor adversarial I1b): NO CIERRA y no pretende; el paquete es honesto y no contradice Conflictos. Sigue Cerrado parcial. || EXT-0 — REABIERTO con argumento nuevo (EXT-M-02, PC-27, PC-25): el «Cerrado parcial» descansaba en que HW/D &lt; 0.75 bajo control de salida fuera un AVISO; el punto se acepta con h_o_fuera_de_rango=True (sin lector fuera de M11) mientras el PasoDeMemoria del mismo punto imprime NO_CUMPLE (SIS-A-07). La v8 §4.3 decide ahora «método no evaluable» por vía Bloqueo, diferible en perfil y no en expediente, nunca cumple=False (subir D sólo baja HW/D, 0.589 → 0.526). Además el paquete I1 decía «M5 no cambia» y EXT-M-01 lo refuta (V1/V2 salen del régimen del barril bajo TW ahogante). La frase elidida de la pág. 3.24 está completa desde EXT-0 (v8 y H_O_CONDICION_TEXTO). Sesiones: EXT-3 (bloqueo, régimen) y E-A (perfil por paso directo). Ficha de decisiones_diferidas.md actualizada. || 43b2531 — EXT-3 (2026-09-20) — CERRADO PARCIAL, con el argumento de EXT-0 resuelto: HW/D &lt; 0.75 bajo control de salida ya NO es un aviso sino `MetodoNoEvaluableError` por vía Bloqueo (diferible en perfil, no en expediente), F4.HO dice DIFERIDO y no NO_CUMPLE, y la compuerta lee el mismo campo (SIS-A-07). V1/V2 salen del régimen del barril (EXT-M-01). Lo ÚNICO que sigue abierto es la tercera condición —que el barril fluya lleno en la mayor parte de su longitud— y con ella el perfil por paso directo (EXT-3b / E-A), con el paquete I1 de H_O_CONDICION_APLICACION intacto.</t>
         </is>
       </c>
     </row>
@@ -14450,7 +14450,7 @@
       </c>
       <c r="L215" s="6" t="inlineStr">
         <is>
-          <t>4141fd5 — La ficha esta obsoleta en LA MITAD de su acusacion --- «no se emite ni al JSON ni al HTML» --- y la otra mitad sigue viva. Al HTML SI llega: `ahogado_por_TW` SI tiene lector de produccion y SI llega a la memoria desde S18 (f865969), dentro del PasoDeMemoria de h_o que emite `M4._pasos_hidraulicos` --- «(manda TW: la salida esta ahogada)» frente a «(manda la aproximacion geometrica)» ---. Se cerro solo, sin que nadie marcara el hallazgo. S19 lo verifica ejecutando las dos ramas, lo escribe en el docstring de `ControlSalida` y lo FIJA con un test sobre el TEXTO RENDERIZADO, no sobre el booleano: hasta ahora el campo asomaba al entregable por una sola frase y nada la protegia. AL JSON NO LLEGA, y eso no se cierra aqui: no llega ninguna pieza del bloque h_o (`grep -n 'h_o' cli.py` esta vacio), ni siquiera los dos flags de condicion de uso. Publicar la etiqueta de la rama sin h_o, TW ni la aproximacion geometrica daria al lector del JSON un veredicto sin los dos numeros que lo producen, que es menos revisable que no publicar nada. Abrir el JSON al bloque h_o ENTERO es una decision propia y no parte de SIS-B-18. Los otros cuatro campos siguen con su decision escrita, como la ficha reconoce. HALLAZGO NUEVO ABIERTO DE PASO: `M9_cabezal.combinaciones()` afirmaba en su docstring que 'M11 la usa' y M11 no la referencia --- corregido, con la razon de por que se conserva. || PRECISADO EN 6b70481: al JSON NO llega, y el cierre anterior daba la ficha por obsoleta entera. Se declara que abrir el JSON al bloque h_o completo es decision propia. || S19d — SHA CORREGIDO. Esta celda citaba el commit de CODIGO de S19b tal como se creo la primera vez: por error estando en `main`, y el texto de la celda se escribio ANTES del cherry-pick que lo llevo a la rama. Al resetear `main` ese commit quedo sin rama, de modo que en un clon limpio NO EXISTE. Su equivalente vivo es 6b70481 --- mismo arbol (`git diff` entre los dos, vacio) y mismo mensaje ---, verificado ancestro de main con `git merge-base --is-ancestor` antes de escribirlo. EL HEX MUERTO NO SE ESCRIBE EN ESTA CELDA, y no es pudor: esta columna es justo lo que lee `verificar_sesion.py`, que no distingue un SHA CITADO de un SHA NOMBRADO de pasada, asi que dejarlo escrito aqui como parte de la explicacion reabre el mismo fallo que la explicacion cierra (probado: 6 fallos se volvieron 20). Regla que queda: en la columna Commit / PR no se escribe un hex que no sea ancestro de main; la arqueologia va al mensaje del commit. Quien necesite el hex muerto lo tiene en el mensaje de 9c00720 («Anotado contra ...») y la correccion entera contada en el de a323bf4. || EXT-3 (2026-09-20) — MITAD JSON CERRADA: el bloque h_o ENTERO viaja a `ResultadoHidraulico` (h_o_m, TW_m, ahogado_por_TW, HW_sobre_D_salida, h_o_fuera_de_rango, h_o_requiere_cautela) y de ahí a `cli._diseno_json` y a `cli.volcar` (línea «h_o :»), junto al régimen y la velocidad de salida y a Q_celda_m3s/numero_celdas (EXT-2-02). La «decisión propia» de abrir el JSON al bloque completo queda tomada. El docstring de `ControlSalida` ya no dice «AL JSON NO LLEGA». La GUI lee el mismo Informe; su tablero de criterios sigue sin mostrar los Bloqueo con criterio=None (PC-03).</t>
+          <t>4141fd5 — La ficha esta obsoleta en LA MITAD de su acusacion --- «no se emite ni al JSON ni al HTML» --- y la otra mitad sigue viva. Al HTML SI llega: `ahogado_por_TW` SI tiene lector de produccion y SI llega a la memoria desde S18 (f865969), dentro del PasoDeMemoria de h_o que emite `M4._pasos_hidraulicos` --- «(manda TW: la salida esta ahogada)» frente a «(manda la aproximacion geometrica)» ---. Se cerro solo, sin que nadie marcara el hallazgo. S19 lo verifica ejecutando las dos ramas, lo escribe en el docstring de `ControlSalida` y lo FIJA con un test sobre el TEXTO RENDERIZADO, no sobre el booleano: hasta ahora el campo asomaba al entregable por una sola frase y nada la protegia. AL JSON NO LLEGA, y eso no se cierra aqui: no llega ninguna pieza del bloque h_o (`grep -n 'h_o' cli.py` esta vacio), ni siquiera los dos flags de condicion de uso. Publicar la etiqueta de la rama sin h_o, TW ni la aproximacion geometrica daria al lector del JSON un veredicto sin los dos numeros que lo producen, que es menos revisable que no publicar nada. Abrir el JSON al bloque h_o ENTERO es una decision propia y no parte de SIS-B-18. Los otros cuatro campos siguen con su decision escrita, como la ficha reconoce. HALLAZGO NUEVO ABIERTO DE PASO: `M9_cabezal.combinaciones()` afirmaba en su docstring que 'M11 la usa' y M11 no la referencia --- corregido, con la razon de por que se conserva. || PRECISADO EN 6b70481: al JSON NO llega, y el cierre anterior daba la ficha por obsoleta entera. Se declara que abrir el JSON al bloque h_o completo es decision propia. || S19d — SHA CORREGIDO. Esta celda citaba el commit de CODIGO de S19b tal como se creo la primera vez: por error estando en `main`, y el texto de la celda se escribio ANTES del cherry-pick que lo llevo a la rama. Al resetear `main` ese commit quedo sin rama, de modo que en un clon limpio NO EXISTE. Su equivalente vivo es 6b70481 --- mismo arbol (`git diff` entre los dos, vacio) y mismo mensaje ---, verificado ancestro de main con `git merge-base --is-ancestor` antes de escribirlo. EL HEX MUERTO NO SE ESCRIBE EN ESTA CELDA, y no es pudor: esta columna es justo lo que lee `verificar_sesion.py`, que no distingue un SHA CITADO de un SHA NOMBRADO de pasada, asi que dejarlo escrito aqui como parte de la explicacion reabre el mismo fallo que la explicacion cierra (probado: 6 fallos se volvieron 20). Regla que queda: en la columna Commit / PR no se escribe un hex que no sea ancestro de main; la arqueologia va al mensaje del commit. Quien necesite el hex muerto lo tiene en el mensaje de 9c00720 («Anotado contra ...») y la correccion entera contada en el de a323bf4. || 43b2531 — EXT-3 (2026-09-20) — MITAD JSON CERRADA: el bloque h_o ENTERO viaja a `ResultadoHidraulico` (h_o_m, TW_m, ahogado_por_TW, HW_sobre_D_salida, h_o_fuera_de_rango, h_o_requiere_cautela) y de ahí a `cli._diseno_json` y a `cli.volcar` (línea «h_o :»), junto al régimen y la velocidad de salida y a Q_celda_m3s/numero_celdas (EXT-2-02). La «decisión propia» de abrir el JSON al bloque completo queda tomada. El docstring de `ControlSalida` ya no dice «AL JSON NO LLEGA». La GUI lee el mismo Informe; su tablero de criterios sigue sin mostrar los Bloqueo con criterio=None (PC-03).</t>
         </is>
       </c>
     </row>
@@ -16202,7 +16202,7 @@
       </c>
       <c r="L246" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-3) (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext3_regimen_barril.py (23, escritos en rojo con xfail strict y liberados al corregir). M4.resolver_control emite el régimen del barril (`modelos.RegimenBarril`: LLENO ⇔ TW ≥ D, PARCIALMENTE_LLENO si no; `M4.regimen_del_barril`) y la velocidad de salida de HDS-5 3.1.6 como Magnitud con procedencia (`M4.velocidad_de_salida`: Q_celda/A(min(D, max(TW, y_c))) bajo control de salida; tirante normal, rama n_min, bajo control de entrada), con el paso F4.REGIMEN y tres citas nuevas (HDS5_3ED.3.1.6#V_SALIDA, #V_SALIDA_TW, HDS5_3ED.3.3.2#V_SALIDA_ENTRADA, verificadas PDF 99-100 y 106). M5: V2 compara la velocidad de la sección efectiva (`V_llena_m_s` = Q_celda/A_llena a barril lleno: 0.0786 m/s &lt; 0.25 en el caso del dictamen), V1 a sección llena no cumple con la cita nueva MC_HHD.4.1.1.3.7b#LLENA (pág. 79, EXIGENCIA); bajo control de salida parcialmente lleno V1/V2 quedan PENDIENTES con `MetodoNoEvaluableError` (`M5._exigir_regimen_evaluable`), diferible en perfil (`cli._verificador_perfil`) y no en expediente; no se inventó criterio de llenado. M6 recibe `ResultadoHidraulico.V_salida`. Dorado cerrado CP12_REGIMEN_LLENO (Q/A_llena, aritmética de la fuente). Línea base: 9 de 13 archivos (README de la línea base, entrada EXT-3). Sin cerrar aquí: el reetiquetado [N]→[A] del 0.75/0.25 (ficha EXT-3-01, sesión EXT-3c) y los dos escenarios de TW para V1/V2 (ficha EXT-3-02).</t>
+          <t>43b2531 — EXT-3 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext3_regimen_barril.py (23, escritos en rojo con xfail strict y liberados al corregir). M4.resolver_control emite el régimen del barril (`modelos.RegimenBarril`: LLENO ⇔ TW ≥ D, PARCIALMENTE_LLENO si no; `M4.regimen_del_barril`) y la velocidad de salida de HDS-5 3.1.6 como Magnitud con procedencia (`M4.velocidad_de_salida`: Q_celda/A(min(D, max(TW, y_c))) bajo control de salida; tirante normal, rama n_min, bajo control de entrada), con el paso F4.REGIMEN y tres citas nuevas (HDS5_3ED.3.1.6#V_SALIDA, #V_SALIDA_TW, HDS5_3ED.3.3.2#V_SALIDA_ENTRADA, verificadas PDF 99-100 y 106). M5: V2 compara la velocidad de la sección efectiva (`V_llena_m_s` = Q_celda/A_llena a barril lleno: 0.0786 m/s &lt; 0.25 en el caso del dictamen), V1 a sección llena no cumple con la cita nueva MC_HHD.4.1.1.3.7b#LLENA (pág. 79, EXIGENCIA); bajo control de salida parcialmente lleno V1/V2 quedan PENDIENTES con `MetodoNoEvaluableError` (`M5._exigir_regimen_evaluable`), diferible en perfil (`cli._verificador_perfil`) y no en expediente; no se inventó criterio de llenado. M6 recibe `ResultadoHidraulico.V_salida`. Dorado cerrado CP12_REGIMEN_LLENO (Q/A_llena, aritmética de la fuente). Línea base: 9 de 13 archivos (README de la línea base, entrada EXT-3). Sin cerrar aquí: el reetiquetado [N]→[A] del 0.75/0.25 (ficha EXT-3-01, sesión EXT-3c) y los dos escenarios de TW para V1/V2 (ficha EXT-3-02).</t>
         </is>
       </c>
     </row>
@@ -16264,7 +16264,7 @@
       </c>
       <c r="L247" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-3) (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext3_regimen_barril.py (23, escritos en rojo con xfail strict y liberados al corregir). `modelos.MetodoNoEvaluableError` (sexta de la taxonomía; `MOTIVO_METODO_NO_EVALUABLE` = «método no evaluable (HDS-5 3.24, Sección 3.5)») viaja como `Bloqueo` con `TipoDeBloqueo.METODO_NO_EVALUABLE`. Compuerta `cli._compuerta_metodo_h_o` tras el bucle de MD, que lee el MISMO campo que juzga el paso F4.HO (`ResultadoHidraulico.h_o_fuera_de_rango`, ya filtrado por control gobernante): diferido a nivel de perfil, bloqueo que impide cerrar a nivel de expediente. F4.HO pasa de NO_CUMPLE a DIFERIDO con el motivo (SIS-A-07: memoria y pipeline dicen lo mismo). Nunca `Verificacion(cumple=False)` ni `DisenoNoFactibleError` por esta causa: `MD.disenar_punto` acumula la excepción como a los pendientes (`_exigir_metodo_evaluable`). B-01 del corredor de referencia: dimensionado CON el bloqueo diferido y el motivo impreso (test_cierre_perfil, test_cli, test_gui_contrato con la ventana real). H_O_CONDICION_APLICACION reescrita («no es un aviso»). Sigue pendiente el perfil por paso directo (EXT-3b / E-A), que deshace la circularidad: NOR-HDS-05 queda Cerrado parcial.</t>
+          <t>43b2531 — EXT-3 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext3_regimen_barril.py (23, escritos en rojo con xfail strict y liberados al corregir). `modelos.MetodoNoEvaluableError` (sexta de la taxonomía; `MOTIVO_METODO_NO_EVALUABLE` = «método no evaluable (HDS-5 3.24, Sección 3.5)») viaja como `Bloqueo` con `TipoDeBloqueo.METODO_NO_EVALUABLE`. Compuerta `cli._compuerta_metodo_h_o` tras el bucle de MD, que lee el MISMO campo que juzga el paso F4.HO (`ResultadoHidraulico.h_o_fuera_de_rango`, ya filtrado por control gobernante): diferido a nivel de perfil, bloqueo que impide cerrar a nivel de expediente. F4.HO pasa de NO_CUMPLE a DIFERIDO con el motivo (SIS-A-07: memoria y pipeline dicen lo mismo). Nunca `Verificacion(cumple=False)` ni `DisenoNoFactibleError` por esta causa: `MD.disenar_punto` acumula la excepción como a los pendientes (`_exigir_metodo_evaluable`). B-01 del corredor de referencia: dimensionado CON el bloqueo diferido y el motivo impreso (test_cierre_perfil, test_cli, test_gui_contrato con la ventana real). H_O_CONDICION_APLICACION reescrita («no es un aviso»). Sigue pendiente el perfil por paso directo (EXT-3b / E-A), que deshace la circularidad: NOR-HDS-05 queda Cerrado parcial.</t>
         </is>
       </c>
     </row>
@@ -17352,7 +17352,7 @@
       </c>
       <c r="L265" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-3) (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext3_regimen_barril.py (23, escritos en rojo con xfail strict y liberados al corregir). `cli._fase_6` pasa a M6 `ResultadoHidraulico.V_salida` (Magnitud, HDS-5 3.1.6): bajo control de salida Q_celda entre el área al tirante min(D, max(TW, y_c)) —1.508 m/s en el caso subcrítico del dictamen, no V_erosion = 1.184—; bajo control de entrada la del tirante normal con n_min (pág. 3.24, «the velocity at normal depth is assumed to be the outlet velocity»). `M6.proteccion_salida(*, V: Magnitud)` imprime la procedencia que trae el número; la clave del JSON de la Fase 6 pasa de V_erosion_m_s a V_salida_m_s. En la línea base B-01 (TW = 1.00 m) recibe 0.112 m/s y d50 baja de 0.126 a 0.0004 m: con la salida ahogada no hay chorro.</t>
+          <t>43b2531 — EXT-3 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext3_regimen_barril.py (23, escritos en rojo con xfail strict y liberados al corregir). `cli._fase_6` pasa a M6 `ResultadoHidraulico.V_salida` (Magnitud, HDS-5 3.1.6): bajo control de salida Q_celda entre el área al tirante min(D, max(TW, y_c)) —1.508 m/s en el caso subcrítico del dictamen, no V_erosion = 1.184—; bajo control de entrada la del tirante normal con n_min (pág. 3.24, «the velocity at normal depth is assumed to be the outlet velocity»). `M6.proteccion_salida(*, V: Magnitud)` imprime la procedencia que trae el número; la clave del JSON de la Fase 6 pasa de V_erosion_m_s a V_salida_m_s. En la línea base B-01 (TW = 1.00 m) recibe 0.112 m/s y d50 baja de 0.126 a 0.0004 m: con la salida ahogada no hay chorro.</t>
         </is>
       </c>
     </row>
@@ -18714,7 +18714,7 @@
       </c>
       <c r="L288" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-3) (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext3_regimen_barril.py (23, escritos en rojo con xfail strict y liberados al corregir). MITAD COMPUERTA: `Bloqueo` vive en `modelos.py` con `tipo: TipoDeBloqueo` (str Enum cuyos valores son los textos que ya imprimía la línea base: CriterioPendienteError, DisenoNoFactibleError, DatoFaltanteError, DatoInvalidoError, LimiteNumericoError, MetodoNoEvaluableError, DiferidoPorAlcance; `TipoDeBloqueo.de_excepcion`), y «fuera de dominio» tiene lector de compuerta (`cli._compuerta_metodo_h_o`) y llega a informe_json y a cli.volcar. `TipoDeVeredicto.DIFERIDO` gana su primer productor de cálculo (F4.HO). QUEDA ABIERTO: unificar `Verificacion.cumple` / `TipoDeVeredicto` / `Bloqueo` en un solo estado de verificación («no aplica» sigue sin existir) y la tupla vacía de `EstabilidadCabezal`.</t>
+          <t>43b2531 — EXT-3 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext3_regimen_barril.py (23, escritos en rojo con xfail strict y liberados al corregir). MITAD COMPUERTA: `Bloqueo` vive en `modelos.py` con `tipo: TipoDeBloqueo` (str Enum cuyos valores son los textos que ya imprimía la línea base: CriterioPendienteError, DisenoNoFactibleError, DatoFaltanteError, DatoInvalidoError, LimiteNumericoError, MetodoNoEvaluableError, DiferidoPorAlcance; `TipoDeBloqueo.de_excepcion`), y «fuera de dominio» tiene lector de compuerta (`cli._compuerta_metodo_h_o`) y llega a informe_json y a cli.volcar. `TipoDeVeredicto.DIFERIDO` gana su primer productor de cálculo (F4.HO). QUEDA ABIERTO: unificar `Verificacion.cumple` / `TipoDeVeredicto` / `Bloqueo` en un solo estado de verificación («no aplica» sigue sin existir) y la tupla vacía de `EstabilidadCabezal`.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cierre(EXT-5): sellos de indice_formulas.md y trazabilidad.csv firmados sobre 149e9bd y SHA en el tracker — 2363 passed, 4 skipped (PyMuPDF sí · ventana Tk sí)
Las cuatro configuraciones se midieron sobre el árbol de 149e9bd:
sí · sí 2363/4; sí · no 2355/12; no · sí 2330/37; no · no 2322/45.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JA9rZZP9yfqTvnqstchwAZ
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -16692,7 +16692,7 @@
       </c>
       <c r="L254" s="6" t="inlineStr">
         <is>
-          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. Validación cerrada: M4._validar_ke (real, finito, `not ke &gt;= 0`) en perdida_carga y en la rama numérica de ke_declarado; declaracion.Procedencia.valor_de_la_celda + difiere_de_la_celda; declarar_desde_tabla exige nota si valor ≠ celda; M11 imprime «DIFIERE de la celda (0.5)». La FORMA (C5-02, clave de fila) queda en EXT-6: ver decisiones_diferidas.md. AUDITOR ADVERSARIAL (EXT-1): refutó la primera versión de la guardia de celda (rechazaba la CLAVE de fila de ke_entrada_cajon declarada por la GUI); corregido en la misma sesión (la celda sólo se cita para valores numéricos) con test de regresión. FORMA (EXT-5, 2026-09-20): Criterio.forma=float para ke_entrada; 'texto', True y [1,2] se rechazan en la puerta con ValueError. La migración a clave de fila (C5-02) sigue en EXT-6.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. Validación cerrada: M4._validar_ke (real, finito, `not ke &gt;= 0`) en perdida_carga y en la rama numérica de ke_declarado; declaracion.Procedencia.valor_de_la_celda + difiere_de_la_celda; declarar_desde_tabla exige nota si valor ≠ celda; M11 imprime «DIFIERE de la celda (0.5)». La FORMA (C5-02, clave de fila) queda en EXT-6: ver decisiones_diferidas.md. AUDITOR ADVERSARIAL (EXT-1): refutó la primera versión de la guardia de celda (rechazaba la CLAVE de fila de ke_entrada_cajon declarada por la GUI); corregido en la misma sesión (la celda sólo se cita para valores numéricos) con test de regresión. FORMA (EXT-5, 2026-09-20, 149e9bd): Criterio.forma=float para ke_entrada; 'texto', True y [1,2] se rechazan en la puerta con ValueError. La migración a clave de fila (C5-02) sigue en EXT-6.</t>
         </is>
       </c>
     </row>
@@ -16816,7 +16816,7 @@
       </c>
       <c r="L256" s="6" t="inlineStr">
         <is>
-          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. establecer_valor_dinamico y escribir_valor_en_archivo rechazan un criterio de resolución Derivada con ValueError («se deriva de &lt;de&gt;; edite sus entradas»); cubre pestaña 2, --declarar y declaracion.declarar_valor. Docstring «DE CUALQUIER CRITERIO» y test «mismo rasero» actualizados. PESTAÑA 2 (EXT-5, 2026-09-20): cara de solo lectura en gui/app.py::_al_seleccionar_criterio — los dos botones que escriben se apagan con el motivo MOTIVO_DERIVADO y el campo ent_valor_declarado se deshabilita; medido en ventana real (tests/apoyo/gui_ext5_real.py).</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. establecer_valor_dinamico y escribir_valor_en_archivo rechazan un criterio de resolución Derivada con ValueError («se deriva de &lt;de&gt;; edite sus entradas»); cubre pestaña 2, --declarar y declaracion.declarar_valor. Docstring «DE CUALQUIER CRITERIO» y test «mismo rasero» actualizados. PESTAÑA 2 (EXT-5, 2026-09-20, 149e9bd): cara de solo lectura en gui/app.py::_al_seleccionar_criterio — los dos botones que escriben se apagan con el motivo MOTIVO_DERIVADO y el campo ent_valor_declarado se deshabilita; medido en ventana real (tests/apoyo/gui_ext5_real.py).</t>
         </is>
       </c>
     </row>
@@ -16878,7 +16878,7 @@
       </c>
       <c r="L257" s="6" t="inlineStr">
         <is>
-          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. Sensibilidad estructurada {campo: (min, max)} evaluada por criterios_adoptados._verificar_dict; 'seccion_receptor' migrado de prosa a dict. Rechaza dict mal formado, claves desconocidas/faltantes, no-real por campo y fuera de rango por campo. FORMA (EXT-5, 2026-09-20): Criterio.forma=dict_con_campos para seccion_receptor y los otros nueve criterios dict; un escalar o un texto se rechaza en la puerta antes de _verificar_dict.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. Sensibilidad estructurada {campo: (min, max)} evaluada por criterios_adoptados._verificar_dict; 'seccion_receptor' migrado de prosa a dict. Rechaza dict mal formado, claves desconocidas/faltantes, no-real por campo y fuera de rango por campo. FORMA (EXT-5, 2026-09-20, 149e9bd): Criterio.forma=dict_con_campos para seccion_receptor y los otros nueve criterios dict; un escalar o un texto se rechaza en la puerta antes de _verificar_dict.</t>
         </is>
       </c>
     </row>
@@ -16940,7 +16940,7 @@
       </c>
       <c r="L258" s="6" t="inlineStr">
         <is>
-          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. M1._exigir_forma_del_mapa: Mapping exterior, filas ∈ CategoriaTR, campos ∈ {R, n}, reales finitos no bool; errata o clave desconocida → DatoInvalidoError con la ruta. Ya no se ignora en silencio. FORMA (EXT-5, 2026-09-20): riesgo_admisible_propietario lleva forma=dict_con_campos; lo que no es un dict se rechaza en la puerta; la forma interior del mapa sigue en M1._exigir_forma_del_mapa.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. M1._exigir_forma_del_mapa: Mapping exterior, filas ∈ CategoriaTR, campos ∈ {R, n}, reales finitos no bool; errata o clave desconocida → DatoInvalidoError con la ruta. Ya no se ignora en silencio. FORMA (EXT-5, 2026-09-20, 149e9bd): riesgo_admisible_propietario lleva forma=dict_con_campos; lo que no es un dict se rechaza en la puerta; la forma interior del mapa sigue en M1._exigir_forma_del_mapa.</t>
         </is>
       </c>
     </row>
@@ -17002,7 +17002,7 @@
       </c>
       <c r="L259" s="6" t="inlineStr">
         <is>
-          <t>EXT-5 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext5_forma_gui.py y tests/apoyo/gui_ext5_real.py. Un solo parser GUI–GUI, gui/componentes.py::interpretar_texto_declarado, usado por ExpedienteApp._interpretar_valor_declarado y VentanaNormativa._valor_tecleado/_validador_de_rango; literal estructurado y literal mal cerrado reciben el mismo veredicto en los dos paneles; la divergencia deliberada con la CLI se conserva con su test (test_gui_contrato).</t>
+          <t>149e9bd — EXT-5 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext5_forma_gui.py y tests/apoyo/gui_ext5_real.py. Un solo parser GUI–GUI, gui/componentes.py::interpretar_texto_declarado, usado por ExpedienteApp._interpretar_valor_declarado y VentanaNormativa._valor_tecleado/_validador_de_rango; literal estructurado y literal mal cerrado reciben el mismo veredicto en los dos paneles; la divergencia deliberada con la CLI se conserva con su test (test_gui_contrato).</t>
         </is>
       </c>
     </row>
@@ -17126,7 +17126,7 @@
       </c>
       <c r="L261" s="6" t="inlineStr">
         <is>
-          <t>EXT-5 (2026-09-20): las seis claves externas entraron a variables_entrada como Poblacion.DATO_EXTERNO (_EXTERNOS); fichas_de_datos_externos derivada del censo para las ocho; GUI de ayuda sin la etiqueta «sin ficha». Ficha EXT-G-03 en decisiones_diferidas.md marcada CERRADA. Estado anterior: a1b4417 — EXT-0 (2026-09-20), Cerrado parcial.</t>
+          <t>149e9bd — EXT-5 (2026-09-20): las seis claves externas entraron a variables_entrada como Poblacion.DATO_EXTERNO (_EXTERNOS); fichas_de_datos_externos derivada del censo para las ocho; GUI de ayuda sin la etiqueta «sin ficha». Ficha EXT-G-03 en decisiones_diferidas.md marcada CERRADA. Estado anterior: a1b4417 — EXT-0 (2026-09-20), Cerrado parcial.</t>
         </is>
       </c>
     </row>
@@ -17912,7 +17912,7 @@
       </c>
       <c r="L274" s="6" t="inlineStr">
         <is>
-          <t>EXT-5 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext5_forma_gui.py y tests/apoyo/gui_ext5_real.py. '1' → int en las dos ventanas; Criterio.forma=int para n_celdas_cajon. El test de ventana real de perfil dejó de ser ciego: afirma n_celdas_cajon == '1' y que C-01 llega a V1/V2; tests/apoyo/gui_ext5_real.py afirma el bloqueo REAL de C-01 (DatoFaltanteError 'S_cauce', único no diferido).</t>
+          <t>149e9bd — EXT-5 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext5_forma_gui.py y tests/apoyo/gui_ext5_real.py. '1' → int en las dos ventanas; Criterio.forma=int para n_celdas_cajon. El test de ventana real de perfil dejó de ser ciego: afirma n_celdas_cajon == '1' y que C-01 llega a V1/V2; tests/apoyo/gui_ext5_real.py afirma el bloqueo REAL de C-01 (DatoFaltanteError 'S_cauce', único no diferido).</t>
         </is>
       </c>
     </row>
@@ -17974,7 +17974,7 @@
       </c>
       <c r="L275" s="6" t="inlineStr">
         <is>
-          <t>EXT-5 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext5_forma_gui.py y tests/apoyo/gui_ext5_real.py. Criterio.forma exigida a las 70 claves por _verificar_criterio (también sin ventana numérica): 'cero' se rechaza en la puerta con ValueError (SIS-E-05) para toda clave de forma no textual; las que aceptan texto son exactamente las de forma str (medido: &lt; 53). 'nan' recibe el mismo veredicto al escribir y al declarar: el parser lo deja como texto, _como_numero rechaza no finitos y validar_contra_rango va en forma MAT-D13 (ConjuntoDeMaximos ya no devuelve AVISO para NaN).</t>
+          <t>149e9bd — EXT-5 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext5_forma_gui.py y tests/apoyo/gui_ext5_real.py. Criterio.forma exigida a las 70 claves por _verificar_criterio (también sin ventana numérica): 'cero' se rechaza en la puerta con ValueError (SIS-E-05) para toda clave de forma no textual; las que aceptan texto son exactamente las de forma str (medido: &lt; 53). 'nan' recibe el mismo veredicto al escribir y al declarar: el parser lo deja como texto, _como_numero rechaza no finitos y validar_contra_rango va en forma MAT-D13 (ConjuntoDeMaximos ya no devuelve AVISO para NaN).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cierre(EXT-6): sellos de indice_formulas.md y trazabilidad.csv firmados sobre 363091b y SHA en el tracker — 2413 passed, 4 skipped (PyMuPDF sí · ventana Tk sí)
El par se midió sobre un checkout limpio de origin/main en 363091b (ext(EXT-6),
fusionado por fast-forward). Las otras tres configuraciones, medidas sobre el
mismo árbol antes del commit: sí · no 2405/12; no · sí 2379/38; no · no
2371/46 — los dos pares sin PyMuPDF suben 49 passed y 1 skipped porque el T5
nuevo del 5.00 m del DG-2018 abre el PDF. Tracker: EXT-N-01, EXT-N-02,
EXT-N-03, EXT-N-04, PC-23, PC-26, PC-30, EXT-G-03 y NOR-HID-02 Cerrados con el
SHA; PC-24 Cerrado parcial → EXT-3c (ficha EXT-6-03). CLAUDE.md: tabla de
cuatro entornos y párrafo de EXT-6.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SZ98SWC6KUQZZWPBuWCLkM
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -4373,17 +4373,17 @@
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
-          <t>Reabierto (EXT-0)</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K42" s="6" t="inlineStr">
         <is>
-          <t>Claude Code (fase1, S12)</t>
+          <t>Claude Code (fase1, S12) → Claude Code (EXT-6)</t>
         </is>
       </c>
       <c r="L42" s="6" t="inlineStr">
         <is>
-          <t>a227cb9+e3f36df+f1b40b2+9822880 — LONG_MAX_CUNETA: pagina impresa 179 (no la que se citaba) y CARACTER POR VALOR, porque las dos cifras no tienen la misma fuerza normativa. Las dos cosas verificadas sobre el PDF. || EXT-0 — REABIERTO (PC-30, EXT-G-03): cierre INCOMPLETO. La cita del registro (MC_HHD_CUNETA) lleva la 179 desde S12, pero lo que la memoria imprime —NUMERAL_FASE_10, Espaciamiento.numeral, la ficha de long_max_cuneta— y la v8 (Fase 10) seguían en 178, más el manifiesto. Verificado en EXT-0 sobre el PDF: la 178 es la Tabla Nº 34; el apartado d) con 250 m y 200 m está en la 179. v8 corregida en EXT-0; textos del código y test contra MC_HHD_CUNETA.pagina_impresa en EXT-6. Ficha nueva en decisiones_diferidas.md (Parte XVI).</t>
+          <t>363091b — EXT-6 (2026-09-20); el cierre con los sellos es el commit siguiente. Cierre completado: los tres textos del codigo a 179 comparados con MC_HHD_CUNETA.pagina_impresa (PC-30). Ficha NOR-HID-02 de decisiones_diferidas.md marcada CERRADA. || Anterior: a227cb9+e3f36df+f1b40b2+9822880 — LONG_MAX_CUNETA: pagina impresa 179 (no la que se citaba) y CARACTER POR VALOR, porque las dos cifras no tienen la misma fuerza normativa. Las dos cosas verificadas sobre el PDF. || EXT-0 — REABIERTO (PC-30, EXT-G-03): cierre INCOMPLETO. La cita del registro (MC_HHD_CUNETA) lleva la 179 desde S12, pero lo que la memoria imprime —NUMERAL_FASE_10, Espaciamiento.numeral, la ficha de long_max_cuneta— y la v8 (Fase 10) seguían en 178, más el manifiesto. Verificado en EXT-0 sobre el PDF: la 178 es la Tabla Nº 34; el apartado d) con 250 m y 200 m está en la 179. v8 corregida en EXT-0; textos del código y test contra MC_HHD_CUNETA.pagina_impresa en EXT-6. Ficha nueva en decisiones_diferidas.md (Parte XVI).</t>
         </is>
       </c>
     </row>
@@ -15966,15 +15966,19 @@
       </c>
       <c r="J242" s="6" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K242" s="6" t="inlineStr">
         <is>
-          <t>pendiente — cadena EXT (docs/planes_mejora/07_CADENA_PROMPTS_EXT.md)</t>
-        </is>
-      </c>
-      <c r="L242" s="6" t="n"/>
+          <t>Claude Code (EXT-6)</t>
+        </is>
+      </c>
+      <c r="L242" s="6" t="inlineStr">
+        <is>
+          <t>363091b — EXT-6 (2026-09-20); el cierre con los sellos es el commit siguiente. Criterio partido: 'edicion_que_rige_el_expediente' (seis fuentes tecnicas de EE.UU.) y 'edicion_legal_que_rige_el_expediente' (Manual de Puentes, derogado por RD 19-2018-MTC/14; la opcion «citada 2016» exige fecha de inicio del expediente y acto verificado del regimen transitorio). Fuente.vigencia (esquema.Vigencia) con acto_aprobatorio/derogado_por en las 16 presentes; T1-01 cerrada. «cuya edicion no la manda nadie» corregido: MP Introduccion (PDF 44) ancla LRFD 2014 7a ed. y permite actualizaciones (cita MP.INTRODUCCION#LRFD_2014, DIS-MP-LRFD-EDICION). Ambos criterios siguen vacios y sin consumidor de calculo. Tests: tests/test_ext6_registro_normativo.py, tests/test_vigencia_fuentes.py.</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="5" t="inlineStr">
@@ -16024,15 +16028,19 @@
       </c>
       <c r="J243" s="6" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K243" s="6" t="inlineStr">
         <is>
-          <t>pendiente — cadena EXT (docs/planes_mejora/07_CADENA_PROMPTS_EXT.md)</t>
-        </is>
-      </c>
-      <c r="L243" s="6" t="n"/>
+          <t>Claude Code (EXT-6)</t>
+        </is>
+      </c>
+      <c r="L243" s="6" t="inlineStr">
+        <is>
+          <t>363091b — EXT-6 (2026-09-20); el cierre con los sellos es el commit siguiente. DG-2018 como Fuente presente (sha1 96ea0442..., 285 pp., Corrida(+1) medido en 284/285; RD 03-2018-MTC/14 verificada por web, no la imprime el ejemplar). Citas 304.07.01, 304.07.02 (+#INCREMENTO, #INCREMENTO_DRENAJE, #T304.09) y 304.10#T304.11; Tablas 304.09 y 304.11 transcritas. Manual de Seguridad Vial 2017 y Manual de Dispositivos censados en PRESENTES_SIN_REGISTRAR con motivo y sha1. Los tres textos corregidos (SIN_FUNDAMENTO F5.V5, talud_terraplen, remanso_derecho_via) y datos_sitio clase_de_via. RNGIV: no se restaura el binario de 5196dd2 (era El Peruano 2006, no el DS 034-2008-MTC); entra como ausente. Ficha EXT-6-01.</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="5" t="inlineStr">
@@ -16082,15 +16090,19 @@
       </c>
       <c r="J244" s="6" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K244" s="6" t="inlineStr">
         <is>
-          <t>pendiente — cadena EXT (docs/planes_mejora/07_CADENA_PROMPTS_EXT.md)</t>
-        </is>
-      </c>
-      <c r="L244" s="6" t="n"/>
+          <t>Claude Code (EXT-6)</t>
+        </is>
+      </c>
+      <c r="L244" s="6" t="inlineStr">
+        <is>
+          <t>363091b — EXT-6 (2026-09-20); el cierre con los sellos es el commit siguiente. norma_producto por (material, forma): M2.norma_producto_de con rotulo explicito para RECTANGULAR («sin norma de producto: marco vaciado in situ (ruta_familia_c §14.1); diseño AASHTO LRFD Sec. 5 y Art. 12.11; construccion EG-2013 503+504; M 259/M 273 ausentes»), anclado en AASHTO_LRFD_9.12.4.2.4 (12-8) y 12.11.1 (12-68); citas de alcance M 170M 1.1 y Note 1, M 36 1.1, A760 1.1; CITA_ALCANCE_NORMA_PRODUCTO; MD._motivo_descarte, M11.rotulo_norma_producto (3 sitios), cli._diseno_json con alcance_norma_producto y CLAVES_DISENO_JSON; AASHTO_M259/M273 en FUENTES_AUSENTES. Linea base de Familia C regenerada: solo texto, ningun numero. Ficha EXT-6-04.</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="5" t="inlineStr">
@@ -16140,17 +16152,17 @@
       </c>
       <c r="J245" s="6" t="inlineStr">
         <is>
-          <t>Cerrado parcial</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K245" s="6" t="inlineStr">
         <is>
-          <t>Claude Code (EXT-0) → EXT-6</t>
+          <t>Claude Code (EXT-0) → Claude Code (EXT-6)</t>
         </is>
       </c>
       <c r="L245" s="6" t="inlineStr">
         <is>
-          <t>a1b4417 — EXT-0 (2026-09-20); el cierre con los sellos es el commit siguiente</t>
+          <t>363091b — EXT-6 (2026-09-20); el cierre con los sellos es el commit siguiente. Citas DG-2018 304.07.01/304.07.02 y Tabla 304.09 en el registro; piso [N] del ancho del derecho de via en constantes_normativas (ANCHO_MIN_DERECHO_VIA_M derivado de la tabla, INCREMENTO_DERECHO_VIA_OBRAS_DRENAJE_M = 5.0), sin consumidor mientras falten 'ancho_derecho_via_m', 'clase_de_via' y el metodo de remanso (ficha EXT-6-02). Estado anterior: a1b4417 — EXT-0 (2026-09-20), Cerrado parcial. || Anterior: a1b4417 — EXT-0 (2026-09-20); el cierre con los sellos es el commit siguiente</t>
         </is>
       </c>
     </row>
@@ -17121,12 +17133,12 @@
       </c>
       <c r="K261" s="6" t="inlineStr">
         <is>
-          <t>Claude Code (EXT-5)</t>
+          <t>Claude Code (EXT-5) → Claude Code (EXT-6)</t>
         </is>
       </c>
       <c r="L261" s="6" t="inlineStr">
         <is>
-          <t>149e9bd — EXT-5 (2026-09-20): las seis claves externas entraron a variables_entrada como Poblacion.DATO_EXTERNO (_EXTERNOS); fichas_de_datos_externos derivada del censo para las ocho; GUI de ayuda sin la etiqueta «sin ficha». Ficha EXT-G-03 en decisiones_diferidas.md marcada CERRADA. Estado anterior: a1b4417 — EXT-0 (2026-09-20), Cerrado parcial.</t>
+          <t>363091b — EXT-6 (2026-09-20); el cierre con los sellos es el commit siguiente. Textos del codigo: F4.MANNING «una geometria con n_max y dos velocidades» (M3 no cambia); M1 columna «TR de diseño» de la tabla de la v8 §2.2, no de la Tabla Nº 02; friccion 47.7 % sobre el termino / 9.6 % sobre H en citas, discrepancias, fuentes, esquema, CN y M4; 178→179 (PC-30). Estado anterior: 149e9bd — EXT-5. || Anterior: 149e9bd — EXT-5 (2026-09-20): las seis claves externas entraron a variables_entrada como Poblacion.DATO_EXTERNO (_EXTERNOS); fichas_de_datos_externos derivada del censo para las ocho; GUI de ayuda sin la etiqueta «sin ficha». Ficha EXT-G-03 en decisiones_diferidas.md marcada CERRADA. Estado anterior: a1b4417 — EXT-0 (2026-09-20), Cerrado parcial.</t>
         </is>
       </c>
     </row>
@@ -18506,15 +18518,19 @@
       </c>
       <c r="J284" s="6" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K284" s="6" t="inlineStr">
         <is>
-          <t>pendiente — cadena EXT (docs/planes_mejora/07_CADENA_PROMPTS_EXT.md)</t>
-        </is>
-      </c>
-      <c r="L284" s="6" t="n"/>
+          <t>Claude Code (EXT-6)</t>
+        </is>
+      </c>
+      <c r="L284" s="6" t="inlineStr">
+        <is>
+          <t>363091b — EXT-6 (2026-09-20); el cierre con los sellos es el commit siguiente. Guardia «PDF presente sin Fuente»: tests/test_ext6_registro_normativo.py::test_todo_pdf_de_normas_es_fuente_presente_o_esta_censado lista normas/*.pdf y exige Fuente presente o censo en fuentes.PRESENTES_SIN_REGISTRAR (esquema.PdfPresenteSinRegistrar, con motivo, sha1 y paginas medidos). RNGIV decidido: no vuelve (ficha EXT-6-01).</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="5" t="inlineStr">
@@ -18569,12 +18585,12 @@
       </c>
       <c r="K285" s="6" t="inlineStr">
         <is>
-          <t>Claude Code (EXT-0) → EXT-3</t>
+          <t>Claude Code (EXT-0) → EXT-3c</t>
         </is>
       </c>
       <c r="L285" s="6" t="inlineStr">
         <is>
-          <t>a1b4417 — EXT-0 (2026-09-20); el cierre con los sellos es el commit siguiente</t>
+          <t>363091b — EXT-6 (2026-09-20); el cierre con los sellos es el commit siguiente. NO se cierra en EXT-6: su resto es la ficha EXT-3-01 (reetiquetar Y_SOBRE_D_MAX y V_MIN, 56 usos en 13 archivos), sesion EXT-3c. Ficha EXT-6-03. || Anterior: a1b4417 — EXT-0 (2026-09-20); el cierre con los sellos es el commit siguiente</t>
         </is>
       </c>
     </row>
@@ -18688,15 +18704,19 @@
       </c>
       <c r="J287" s="6" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K287" s="6" t="inlineStr">
         <is>
-          <t>pendiente — cadena EXT (docs/planes_mejora/07_CADENA_PROMPTS_EXT.md)</t>
-        </is>
-      </c>
-      <c r="L287" s="6" t="n"/>
+          <t>Claude Code (EXT-6)</t>
+        </is>
+      </c>
+      <c r="L287" s="6" t="inlineStr">
+        <is>
+          <t>363091b — EXT-6 (2026-09-20); el cierre con los sellos es el commit siguiente. Ventana partida en legal (MP) y tecnica (seis de EE.UU.); ver EXT-N-01.</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="5" t="inlineStr">
@@ -18932,17 +18952,17 @@
       </c>
       <c r="J291" s="6" t="inlineStr">
         <is>
-          <t>Cerrado parcial</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K291" s="6" t="inlineStr">
         <is>
-          <t>Claude Code (EXT-0) → EXT-6</t>
+          <t>Claude Code (EXT-0) → Claude Code (EXT-6)</t>
         </is>
       </c>
       <c r="L291" s="6" t="inlineStr">
         <is>
-          <t>a1b4417 — EXT-0 (2026-09-20); el cierre con los sellos es el commit siguiente</t>
+          <t>363091b — EXT-6 (2026-09-20); el cierre con los sellos es el commit siguiente. NUMERAL_FASE_10 lee MC_HHD_CUNETA.pagina_impresa; Espaciamiento.numeral y long_max_cuneta.fuente a 179; test_la_pagina_de_la_cuneta_que_imprime_la_memoria_es_la_del_registro los compara con la cita. Estado anterior: a1b4417 — EXT-0, Cerrado parcial. || Anterior: a1b4417 — EXT-0 (2026-09-20); el cierre con los sellos es el commit siguiente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cierre(EXT-7): sellos de indice_formulas.md y trazabilidad.csv firmados sobre 42a1cb1, SHA en el tracker y tabla de cuatro entornos — 2471 passed, 4 skipped (PyMuPDF sí · ventana Tk sí)
Las cuatro configuraciones medidas en serie sobre origin/main en 42a1cb1:
sí·sí 2471/4, sí·no 2463/12, no·sí 2437/38, no·no 2429/46 (+58 exactos
sobre EXT-6). CLAUDE.md: párrafo de EXT-7 en la sección de tests, tabla,
recuento 2475 y 73 criterios.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015yJG3sCBFAAaUEGT2sqBmo
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -16472,7 +16472,7 @@
       </c>
       <c r="L250" s="6" t="inlineStr">
         <is>
-          <t>SHA: ver commit de cierre — EXT-7 (2026-09-20). `M9.cuantia_de_diseno` y `M9.verificar_cuantia` (argumento `cortante_alto` obligatorio en las dos) leen, con cortante alto, primero el PLANO del cortante ('regimen_cortante_muro_e060_art_11_10_2', categoria en_el_plano / perpendicular_al_plano, [A] expediente, vacio: 11.10.2 vs 11.10.1 -&gt; 11.12) y despues el piso de la direccion: horizontal 'cortante_alto_muro_e060_art_11_10_10_2', vertical el criterio nuevo 'cuantia_vertical_cortante_alto_e060_art_11_10_10_3' ([A] expediente, vacio, resolucion que nombra hm, lm y la rho_h requerida por 11.10.10.1). La rama vertical DETIENE con CriterioPendienteError en vez de devolver 0.0015; con regimen perpendicular ni 11.10.10.2 ni .3 rigen y el numeral lo dice. Docstring corregido (la afirmacion negativa falsa ya no esta en el modulo; test por AST). La ec. (11-32) NO se implementa (EXT-7-01 en decisiones_diferidas.md). Tests: tests/test_ext7_cabezal.py (bloque M-05, parametrizado en vertical y horizontal).</t>
+          <t>42a1cb1 — EXT-7 (2026-09-20); el cierre con los sellos es el commit siguiente. `M9.cuantia_de_diseno` y `M9.verificar_cuantia` (argumento `cortante_alto` obligatorio en las dos) leen, con cortante alto, primero el PLANO del cortante ('regimen_cortante_muro_e060_art_11_10_2', categoria en_el_plano / perpendicular_al_plano, [A] expediente, vacio: 11.10.2 vs 11.10.1 -&gt; 11.12) y despues el piso de la direccion: horizontal 'cortante_alto_muro_e060_art_11_10_10_2', vertical el criterio nuevo 'cuantia_vertical_cortante_alto_e060_art_11_10_10_3' ([A] expediente, vacio, resolucion que nombra hm, lm y la rho_h requerida por 11.10.10.1). La rama vertical DETIENE con CriterioPendienteError en vez de devolver 0.0015; con regimen perpendicular ni 11.10.10.2 ni .3 rigen y el numeral lo dice. Docstring corregido (la afirmacion negativa falsa ya no esta en el modulo; test por AST). La ec. (11-32) NO se implementa (EXT-7-01 en decisiones_diferidas.md). Tests: tests/test_ext7_cabezal.py (bloque M-05, parametrizado en vertical y horizontal).</t>
         </is>
       </c>
     </row>
@@ -16534,7 +16534,7 @@
       </c>
       <c r="L251" s="6" t="inlineStr">
         <is>
-          <t>SHA: ver commit de cierre — EXT-7 (2026-09-20). `M9.empujes_trasdos` calcula el empuje estatico Y la sobrecarga con el Ka de Coulomb del Manual (`k_a_coulomb`, los cuatro angulos de Sec. 9.2 tambien en condicion ESTATICA; un vacio detiene). Cita nueva verificada MP.2.4.4.1.5.3 (pag. impresa 135 / PDF 136, PERMISO «se puede tomar como»); discrepancia DIS-HR-KA-COULOMB registrada RESUELTA (v8 §9.2 enmendada en EXT-0); declarada en el punto de uso (docstring, `EmpujesTrasdos.numeral_k_a`) y en la memoria (`KA_COULOMB_DECLARACION` por `condicion_normativa_cabezal`). `ka_rankine` se conserva como patron del caso limite. Bloque C de CP9_EMPUJE_TRASDOS con i = 5, beta = 5, delta = 17 grados dentro de las ventanas (Coulomb +9.67 % sobre Rankine), recomputado en el __main__ con la escritura del Manual (theta desde la horizontal). Sensibilidad de 'pendiente_relleno_trasdos_i': con k_h = 0.50 (psi = 26.6) M-O solo tiene solucion para i &lt; phi - psi (3.4 grados con phi = 30, 8.4 con phi = 35). Se adopto Coulomb entero, no la guardia minima (EXT-7-03). Auditoria adversarial de EXT-7: (a) el rango «-6.25 % a +7.23 %» de la columna Hallazgo (y de la enmienda de EXT-0 en la v8) es FALSO: medido con k_a_coulomb sobre las cuatro ventanas, de -11.1 % (phi = 30, i = beta = 0, delta = 22.7) a +44.4 % (phi = 38, i = beta = 10, delta = 0); la v8 §9.2 lleva la corrección (bloque «Corregido (EXT-M-06, EXT-7)»); (b) la resultante de Coulomb actúa a delta + beta de la horizontal y el cálculo la toma entera como horizontal: declarado en empujes_trasdos y en la memoria con su dirección (conservador para E2/E3, no para E1 en la componente vertical), descomposición diferida en EXT-7-04.</t>
+          <t>42a1cb1 — EXT-7 (2026-09-20); el cierre con los sellos es el commit siguiente. `M9.empujes_trasdos` calcula el empuje estatico Y la sobrecarga con el Ka de Coulomb del Manual (`k_a_coulomb`, los cuatro angulos de Sec. 9.2 tambien en condicion ESTATICA; un vacio detiene). Cita nueva verificada MP.2.4.4.1.5.3 (pag. impresa 135 / PDF 136, PERMISO «se puede tomar como»); discrepancia DIS-HR-KA-COULOMB registrada RESUELTA (v8 §9.2 enmendada en EXT-0); declarada en el punto de uso (docstring, `EmpujesTrasdos.numeral_k_a`) y en la memoria (`KA_COULOMB_DECLARACION` por `condicion_normativa_cabezal`). `ka_rankine` se conserva como patron del caso limite. Bloque C de CP9_EMPUJE_TRASDOS con i = 5, beta = 5, delta = 17 grados dentro de las ventanas (Coulomb +9.67 % sobre Rankine), recomputado en el __main__ con la escritura del Manual (theta desde la horizontal). Sensibilidad de 'pendiente_relleno_trasdos_i': con k_h = 0.50 (psi = 26.6) M-O solo tiene solucion para i &lt; phi - psi (3.4 grados con phi = 30, 8.4 con phi = 35). Se adopto Coulomb entero, no la guardia minima (EXT-7-03). Auditoria adversarial de EXT-7: (a) el rango «-6.25 % a +7.23 %» de la columna Hallazgo (y de la enmienda de EXT-0 en la v8) es FALSO: medido con k_a_coulomb sobre las cuatro ventanas, de -11.1 % (phi = 30, i = beta = 0, delta = 22.7) a +44.4 % (phi = 38, i = beta = 10, delta = 0); la v8 §9.2 lleva la corrección (bloque «Corregido (EXT-M-06, EXT-7)»); (b) la resultante de Coulomb actúa a delta + beta de la horizontal y el cálculo la toma entera como horizontal: declarado en empujes_trasdos y en la memoria con su dirección (conservador para E2/E3, no para E1 en la componente vertical), descomposición diferida en EXT-7-04.</t>
         </is>
       </c>
     </row>
@@ -16596,7 +16596,7 @@
       </c>
       <c r="L252" s="6" t="inlineStr">
         <is>
-          <t>SHA: ver commit de cierre — EXT-7 (2026-09-20). `modelos.EstabilidadCabezal` lleva `exigidas` (derivadas de `constantes_normativas.FS` por `FS_CODIGO`, E1..E5; `M9.EXIGIDAS_SEC_9_3`), `__post_init__` que rechaza con ValueError el conjunto vacio, las `exigidas` vacias o repetidas, un codigo fuera de las exigidas, un codigo repetido y un motivo de pendiente sobre una presente; `estabilidad_interna_cumple` (lo que `estable` afirmaba antes, con su nombre), `pendientes` y `estable` solo con todas las exigidas presentes y cumplidas; `motivos_pendientes` (codigo, clave). `verificar_estabilidad` registra E4/E5 como pendientes de 'metodo_estabilidad_global' y admite `exigidas` ampliado (E6, probado). E6 no entra por defecto: EXT-7-02 en decisiones_diferidas.md. Los dos tests que pineaban `estable` con tres items se reescribieron (test_M9_cabezal). Sin lector productivo: nada se cablea a la CLI.</t>
+          <t>42a1cb1 — EXT-7 (2026-09-20); el cierre con los sellos es el commit siguiente. `modelos.EstabilidadCabezal` lleva `exigidas` (derivadas de `constantes_normativas.FS` por `FS_CODIGO`, E1..E5; `M9.EXIGIDAS_SEC_9_3`), `__post_init__` que rechaza con ValueError el conjunto vacio, las `exigidas` vacias o repetidas, un codigo fuera de las exigidas, un codigo repetido y un motivo de pendiente sobre una presente; `estabilidad_interna_cumple` (lo que `estable` afirmaba antes, con su nombre), `pendientes` y `estable` solo con todas las exigidas presentes y cumplidas; `motivos_pendientes` (codigo, clave). `verificar_estabilidad` registra E4/E5 como pendientes de 'metodo_estabilidad_global' y admite `exigidas` ampliado (E6, probado). E6 no entra por defecto: EXT-7-02 en decisiones_diferidas.md. Los dos tests que pineaban `estable` con tres items se reescribieron (test_M9_cabezal). Sin lector productivo: nada se cablea a la CLI.</t>
         </is>
       </c>
     </row>
@@ -19342,7 +19342,7 @@
       </c>
       <c r="L297" s="6" t="inlineStr">
         <is>
-          <t>SHA: ver commit de cierre — EXT-7 (2026-09-20). Cerrado con EXT-M-05: la rama vertical con cortante alto se detiene en 'cuantia_vertical_cortante_alto_e060_art_11_10_10_3' (y antes en el plano del cortante, 'regimen_cortante_muro_e060_art_11_10_2'); la afirmacion negativa falsa del docstring se retiro y un test por AST comprueba que M9 no la contiene ni opera con hm/lm. La ec. (11-32) no se implementa (EXT-7-01).</t>
+          <t>42a1cb1 — EXT-7 (2026-09-20); el cierre con los sellos es el commit siguiente. Cerrado con EXT-M-05: la rama vertical con cortante alto se detiene en 'cuantia_vertical_cortante_alto_e060_art_11_10_10_3' (y antes en el plano del cortante, 'regimen_cortante_muro_e060_art_11_10_2'); la afirmacion negativa falsa del docstring se retiro y un test por AST comprueba que M9 no la contiene ni opera con hm/lm. La ec. (11-32) no se implementa (EXT-7-01).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cierre(EXT-8): sellos de indice_formulas.md y trazabilidad.csv firmados sobre 8c1ac25, SHA en el tracker y tabla de cuatro entornos — 2511 passed, 4 skipped (PyMuPDF sí · ventana Tk sí)
Las cuatro configuraciones medidas en serie sobre un checkout limpio de
origin/main en 8c1ac25: sí·sí 2511/4, sí·no 2502/13 (sin DISPLAY y con un
xvfb-run que falla), no·sí 2476/39 y no·no 2467/48 (PyMuPDF desinstalado y
reinstalado). collected = 2515 en las cuatro.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBQxwVdyW3m3cGwxMRY8MW
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -17762,7 +17762,7 @@
       </c>
       <c r="L271" s="6" t="inlineStr">
         <is>
-          <t>EXT-8 (2026-09-20), commit ext(EXT-8) — el SHA se escribe en el commit de cierre siguiente. `import cli` pasó de 870–930 ms a 125–150 ms (medido con -X importtime, mínimo de tres corridas): weasyprint perezoso dentro de `M11.weasyprint_disponible()`/`exportar_pdf` (conserva `WeasyHTML`, `FALLO_WEASYPRINT`, `WEASYPRINT_AUSENTE` y el diagnóstico ImportError vs OSError); `scipy.optimize.brentq` importado en el punto de uso (M3, M4); `variables_entrada.VARIABLES` perezoso por `__getattr__` de módulo con la guardia `_coherencia_del_censo` en el primer acceso. Tests: tests/test_ext8_rendimiento_gui.py (bloque PC-10: presupuesto &lt; 0.3 s en subproceso, nada cargado tras `import cli`, sonda con los dos diagnósticos).</t>
+          <t>EXT-8 (2026-09-20), commit 8c1ac25 — ext(EXT-8); el cierre con los sellos es el commit siguiente. `import cli` pasó de 870–930 ms a 125–150 ms (medido con -X importtime, mínimo de tres corridas): weasyprint perezoso dentro de `M11.weasyprint_disponible()`/`exportar_pdf` (conserva `WeasyHTML`, `FALLO_WEASYPRINT`, `WEASYPRINT_AUSENTE` y el diagnóstico ImportError vs OSError); `scipy.optimize.brentq` importado en el punto de uso (M3, M4); `variables_entrada.VARIABLES` perezoso por `__getattr__` de módulo con la guardia `_coherencia_del_censo` en el primer acceso. Tests: tests/test_ext8_rendimiento_gui.py (bloque PC-10: presupuesto &lt; 0.3 s en subproceso, nada cargado tras `import cli`, sonda con los dos diagnósticos).</t>
         </is>
       </c>
     </row>
@@ -17824,7 +17824,7 @@
       </c>
       <c r="L272" s="6" t="inlineStr">
         <is>
-          <t>EXT-8 (2026-09-20), commit ext(EXT-8) — el SHA se escribe en el commit de cierre siguiente. PDF por SUBPROCESO: `gui/exportacion_pdf.ProcesoPdf` corre, con la sesión de LA CORRIDA (`sesion_de_la_corrida`: entradas fotografiadas al correr y criterios del `ContextoCorrida` congelado, no los campos vivos — auditor adversarial), `cli.py --sesion &lt;sesión serializada&gt; --pdf … --json &lt;aparte&gt; --plantilla … --progreso`; `cli --sesion` repone proyecto, CSV, externos, alcance y criterios CON procedencia por `declaracion.restaurar_sesion` (esquema único en `src/sesion.py`, reexportado por la GUI); progreso por líneas `progreso: hecho/total etapa` de stdout leídas desde `after` (sin hilo); «Cancelar PDF» termina el proceso; botón apagado con `MOTIVO_EXPORTANDO_PDF` y rótulo; estado terminal en `lbl_estado_pdf`; ayuda del botón con el límite medido y vía navegador ofrecida por encima de `UMBRAL_PUNTOS_PDF` (40). Contrato `M11.WeasyHTML` conservado (los tests siguen parcheándolo). Equivalencia medida: mismo JSON por las dos puertas salvo la marca de tiempo (ficha EXT-8-02; EXT-8-03 para las claves enteras). Tests: test_ext8_rendimiento_gui.py (bloque PC-11) y ventana real tests/apoyo/gui_ext8_real.py.</t>
+          <t>EXT-8 (2026-09-20), commit 8c1ac25 — ext(EXT-8); el cierre con los sellos es el commit siguiente. PDF por SUBPROCESO: `gui/exportacion_pdf.ProcesoPdf` corre, con la sesión de LA CORRIDA (`sesion_de_la_corrida`: entradas fotografiadas al correr y criterios del `ContextoCorrida` congelado, no los campos vivos — auditor adversarial), `cli.py --sesion &lt;sesión serializada&gt; --pdf … --json &lt;aparte&gt; --plantilla … --progreso`; `cli --sesion` repone proyecto, CSV, externos, alcance y criterios CON procedencia por `declaracion.restaurar_sesion` (esquema único en `src/sesion.py`, reexportado por la GUI); progreso por líneas `progreso: hecho/total etapa` de stdout leídas desde `after` (sin hilo); «Cancelar PDF» termina el proceso; botón apagado con `MOTIVO_EXPORTANDO_PDF` y rótulo; estado terminal en `lbl_estado_pdf`; ayuda del botón con el límite medido y vía navegador ofrecida por encima de `UMBRAL_PUNTOS_PDF` (40). Contrato `M11.WeasyHTML` conservado (los tests siguen parcheándolo). Equivalencia medida: mismo JSON por las dos puertas salvo la marca de tiempo (ficha EXT-8-02; EXT-8-03 para las claves enteras). Tests: test_ext8_rendimiento_gui.py (bloque PC-11) y ventana real tests/apoyo/gui_ext8_real.py.</t>
         </is>
       </c>
     </row>
@@ -17886,7 +17886,7 @@
       </c>
       <c r="L273" s="6" t="inlineStr">
         <is>
-          <t>EXT-8 (2026-09-20), commit ext(EXT-8) — el SHA se escribe en el commit de cierre siguiente. F2.LUZ una vez por punto (`M11.desarrollo_de_verificaciones`, compartida con `traza_punto`); punteros como enlaces (`ancla_de_discrepancia`, `ancla_de_criterio`); anexo único `M11.anexo_referencias` con anclas por cita_id (`ancla_de_cita`, `ancla_de_fundamento`, `ancla_de_umbral`), textos de `Registro`; `memoria_html_por_partes` (streaming) y `exportar_html` escribiendo por trozos; progreso por punto. MEDIDO: 54.0 KB → 44.6 KB y ~20 → 14.0 páginas marginales por punto; repetición 44 % → 7 %. El objetivo &lt; 15 KB / &lt; 10 páginas NO se alcanzó: lo que queda es contenido del punto (decisión explícita frente a §4.4 en la ficha EXT-8-01). Techos fijados sobre la medida en test_ext8_rendimiento_gui.py. Línea base de la Familia C regenerada (formato de la memoria; ningún número de cálculo se mueve).</t>
+          <t>EXT-8 (2026-09-20), commit 8c1ac25 — ext(EXT-8); el cierre con los sellos es el commit siguiente. F2.LUZ una vez por punto (`M11.desarrollo_de_verificaciones`, compartida con `traza_punto`); punteros como enlaces (`ancla_de_discrepancia`, `ancla_de_criterio`); anexo único `M11.anexo_referencias` con anclas por cita_id (`ancla_de_cita`, `ancla_de_fundamento`, `ancla_de_umbral`), textos de `Registro`; `memoria_html_por_partes` (streaming) y `exportar_html` escribiendo por trozos; progreso por punto. MEDIDO: 54.0 KB → 44.6 KB y ~20 → 14.0 páginas marginales por punto; repetición 44 % → 7 %. El objetivo &lt; 15 KB / &lt; 10 páginas NO se alcanzó: lo que queda es contenido del punto (decisión explícita frente a §4.4 en la ficha EXT-8-01). Techos fijados sobre la medida en test_ext8_rendimiento_gui.py. Línea base de la Familia C regenerada (formato de la memoria; ningún número de cálculo se mueve).</t>
         </is>
       </c>
     </row>
@@ -18196,7 +18196,7 @@
       </c>
       <c r="L278" s="6" t="inlineStr">
         <is>
-          <t>EXT-8 (2026-09-20), commit ext(EXT-8) — el SHA se escribe en el commit de cierre siguiente. `gui/componentes.py`: `unidades_de_rueda` (Windows ±120, macOS deltas pequeños, X11 Button-4/5) y `MarcoScroll.EVENTOS_RUEDA`; `BotonAccion.con_rotulo` (rótulo visible con el mismo motivo que el tooltip; la fila de exportadores lo usa); Escape cierra `VentanaNormativa`, `VentanaAyudaEntrada` y la traza; Control-Return ejecuta (`ExpedienteApp._crear_interfaz`). Tests: test_ext8_rendimiento_gui.py (bloque PC-17) y ventana real tests/apoyo/gui_ext8_real.py.</t>
+          <t>EXT-8 (2026-09-20), commit 8c1ac25 — ext(EXT-8); el cierre con los sellos es el commit siguiente. `gui/componentes.py`: `unidades_de_rueda` (Windows ±120, macOS deltas pequeños, X11 Button-4/5) y `MarcoScroll.EVENTOS_RUEDA`; `BotonAccion.con_rotulo` (rótulo visible con el mismo motivo que el tooltip; la fila de exportadores lo usa); Escape cierra `VentanaNormativa`, `VentanaAyudaEntrada` y la traza; Control-Return ejecuta (`ExpedienteApp._crear_interfaz`). Tests: test_ext8_rendimiento_gui.py (bloque PC-17) y ventana real tests/apoyo/gui_ext8_real.py.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cierre(EXT-11): tabla de cuatro entornos medida sobre e734c23, sellos de trazabilidad e índice de fórmulas y SHA en el tracker — 3776 passed, 3 skipped (PyMuPDF sí · ventana Tk sí)
Las cuatro configuraciones, en serie, sobre un git worktree limpio de
e734c23 (origin/main tras el fast-forward; las dos sin Tk sin DISPLAY y
con un xvfb-run que falla; las dos sin PyMuPDF desinstalandolo y
reinstalandolo):

  PyMuPDF si · Tk si  3776 passed,  3 skipped
  PyMuPDF si · Tk no  3766 passed, 13 skipped
  PyMuPDF no · Tk si  3741 passed, 38 skipped
  PyMuPDF no · Tk no  3731 passed, 48 skipped

collected = 3779 en las cuatro (2617 + 1162). Sellos de trazabilidad.csv
e indice_formulas.md regenerados con ese par (manifiesto_citas.md no
cambia de cuerpo). Tracker: las cinco filas de EXT-11 citan e734c23.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B2e6gcxvQFas4mf5yPUPwZ
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -18266,7 +18266,7 @@
       </c>
       <c r="L279" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-11) — SHA en el commit de cierre — EXT-11 (2026-09-21): residuo cerrado. La línea base deja de ser la única defensa de EXT-M-01..M-04: siete propiedades por mallas en tests/test_ext11_propiedades.py (Q = V_sedimentación·A en circular y rectangular; Q_total = N·Q_celda a través de MD→M4; V_erosion ≥ V_sedimentación; continuidad y linealidad de la transición en las dos formas; monotonía de HW(Q) bajo Forma 1; tirante_normal = None para Q ≥ Q_lleno; HW(N=3) ≠ HW(N=1) y HW(N, N·Q) = HW(1, Q)). La ceguera a M-03 «por construcción» queda cubierta por P2/P7, que pasan por MD.disenar_material → M4.caudal_por_celda. Mutación medida con tests/apoyo/mutacion.py: 679 mutantes generados por AST sobre M3–M5/MD, M2._par_de_manning y las tres propiedades del par de n; primera vuelta contra diez archivos objetivo: 568 muertos (83.6 %); segunda vuelta (línea base, cierre de perfil, CLI) sobre los 111 restantes: 65 muertos; 46 vivos, 43 tras los tests de la segunda tanda; sin las propiedades ni los tests que la mutación motivó, la primera vuelta daba 489/679 (72.0 %) sobre los ocho archivos objetivo originales. Censo de supervivientes con razón en tests/test_ext11_mutacion.py. Sin hypothesis/mutmut (consulta sin respuesta: ficha EXT-11-01).</t>
+          <t>e734c23 — EXT-11 (2026-09-21): residuo cerrado. La línea base deja de ser la única defensa de EXT-M-01..M-04: siete propiedades por mallas en tests/test_ext11_propiedades.py (Q = V_sedimentación·A en circular y rectangular; Q_total = N·Q_celda a través de MD→M4; V_erosion ≥ V_sedimentación; continuidad y linealidad de la transición en las dos formas; monotonía de HW(Q) bajo Forma 1; tirante_normal = None para Q ≥ Q_lleno; HW(N=3) ≠ HW(N=1) y HW(N, N·Q) = HW(1, Q)). La ceguera a M-03 «por construcción» queda cubierta por P2/P7, que pasan por MD.disenar_material → M4.caudal_por_celda. Mutación medida con tests/apoyo/mutacion.py: 679 mutantes generados por AST sobre M3–M5/MD, M2._par_de_manning y las tres propiedades del par de n; primera vuelta contra diez archivos objetivo: 568 muertos (83.6 %); segunda vuelta (línea base, cierre de perfil, CLI) sobre los 111 restantes: 65 muertos; 46 vivos, 43 tras los tests de la segunda tanda; sin las propiedades ni las tandas que la mutación motivó: 504/679 (74.2 %), y 64 mutantes mueren sólo por ellas. Censo de supervivientes con razón en tests/test_ext11_mutacion.py. Sin hypothesis/mutmut (consulta sin respuesta: ficha EXT-11-01).</t>
         </is>
       </c>
     </row>
@@ -18390,7 +18390,7 @@
       </c>
       <c r="L281" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-11) — SHA en el commit de cierre — EXT-11 (2026-09-21): `informe_dimensionado` de test_cli es una corrida REAL: la de perfil con las entradas de la línea base dimensiona A-01, A-02 y B-01 en concreto reforzado (D 0.90/0.90/1.05 m, Fases 6 y 7 reales) y la de expediente recibe esos resultados del producto para que la Fase 8 corra sobre ellos (cama de apoyo real, bloqueo real en clases_producto_por_relleno). El stub HDPE D = 0.60 m se retiró; queda un solo doble de la capa de reporte (`informe_con_criterio_desconocido`). Por qué no se dimensiona en expediente sin ayuda: ficha EXT-11-04.</t>
+          <t>e734c23 — EXT-11 (2026-09-21): `informe_dimensionado` de test_cli es una corrida REAL: la de perfil con las entradas de la línea base dimensiona A-01, A-02 y B-01 en concreto reforzado (D 0.90/0.90/1.05 m, Fases 6 y 7 reales) y la de expediente recibe esos resultados del producto para que la Fase 8 corra sobre ellos (cama de apoyo real, bloqueo real en clases_producto_por_relleno). El stub HDPE D = 0.60 m se retiró; queda un solo doble de la capa de reporte (`informe_con_criterio_desconocido`). Por qué no se dimensiona en expediente sin ayuda: ficha EXT-11-04.</t>
         </is>
       </c>
     </row>
@@ -18452,7 +18452,7 @@
       </c>
       <c r="L282" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-11) — SHA en el commit de cierre — EXT-11 (2026-09-21): test_anticipo cuenta los nodos `Name` de VERIFICACIONES_DIFERIDAS_POR_ALCANCE por AST; test_gui_contrato busca la llamada `trace_add('write', …)` dentro de CampoValidable por AST; test_ext8 pasa dos presencias más al AST. Guardia nueva en test_guardias_de_la_suite (`afirmaciones_textuales_sobre_codigo`): `getsource(...).count(` y `"x" in &lt;ruta .py&gt;.read_text()` sin ast.parse en la misma función fallan, salvo los 7 sitios del censo TEXTUAL_CON_RAZON (ausencia de una frase, presencia de un comentario, ancla de reescritura, rótulo de la GUI, nombre de archivo en una tupla), comprobado en las dos direcciones y con cuatro autopruebas del detector.</t>
+          <t>e734c23 — EXT-11 (2026-09-21): test_anticipo cuenta los nodos `Name` de VERIFICACIONES_DIFERIDAS_POR_ALCANCE por AST; test_gui_contrato busca la llamada `trace_add('write', …)` dentro de CampoValidable por AST; test_ext8 pasa dos presencias más al AST. Guardia nueva en test_guardias_de_la_suite (`afirmaciones_textuales_sobre_codigo`): `getsource(...).count(` y `"x" in &lt;ruta .py&gt;.read_text()` sin ast.parse en la misma función fallan, salvo los 7 sitios del censo TEXTUAL_CON_RAZON (ausencia de una frase, presencia de un comentario, ancla de reescritura, rótulo de la GUI, nombre de archivo en una tupla), comprobado en las dos direcciones y con cuatro autopruebas del detector.</t>
         </is>
       </c>
     </row>
@@ -18514,7 +18514,7 @@
       </c>
       <c r="L283" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-11) — SHA en el commit de cierre — EXT-11 (2026-09-21): (1) test_MD: el skip permanente se sustituyó por la ausencia REAL de M5 en un subproceso sobre una copia del árbol sin el archivo (la suite pasa de 4 a 3 saltos en sí·sí); (2) test_bandera_pdf marcado `lento` (marca registrada en conftest; 12.8 s medidos en 5196dd2 y en EXT-11; no se salta); (3) test_linea_base: el determinismo se demuestra contra los archivos comprometidos y la segunda corrida (6 s) sólo se lanza en rojo (ficha EXT-11-05); la fixture de módulo ya compartía la corrida entre los otros tres tests; (4) censo PUBLICAS_SIN_REFERENCIA_EN_TESTS en test_guardias_de_la_suite: 23 hoy (16 en 5196dd2; la suite creció), cada una con su consumidor de producción comprobado por AST, fijado en las dos direcciones. Medido en 5196dd2 con --durations: bandera_pdf 12.8 s, T3 jerarquía 9.5 s, línea base 6.1 + 6.0 s.</t>
+          <t>e734c23 — EXT-11 (2026-09-21): (1) test_MD: el skip permanente se sustituyó por la ausencia REAL de M5 en un subproceso sobre una copia del árbol sin el archivo (la suite pasa de 4 a 3 saltos en sí·sí); (2) test_bandera_pdf marcado `lento` (marca registrada en conftest; 12.8 s medidos en 5196dd2 y en EXT-11; no se salta); (3) test_linea_base: el determinismo se demuestra contra los archivos comprometidos y la segunda corrida (6 s) sólo se lanza en rojo (ficha EXT-11-05); la fixture de módulo ya compartía la corrida entre los otros tres tests; (4) censo PUBLICAS_SIN_REFERENCIA_EN_TESTS en test_guardias_de_la_suite: 23 hoy (16 en 5196dd2; la suite creció), cada una con su consumidor de producción comprobado por AST, fijado en las dos direcciones. Medido en 5196dd2 con --durations: bandera_pdf 12.8 s, T3 jerarquía 9.5 s, línea base 6.1 + 6.0 s.</t>
         </is>
       </c>
     </row>
@@ -18948,7 +18948,7 @@
       </c>
       <c r="L290" s="6" t="inlineStr">
         <is>
-          <t>ext(EXT-11) — SHA en el commit de cierre — EXT-11 (2026-09-21): el cruce como test en tests/test_ext11_cruce_temarios.py: 71 ítems ALTA/CRÍTICA (severidad final si hay veredicto, propuesta si no), 26 cubiertos por fila propia o mención en el tracker y 45 por el censo CUBIERTOS_POR_FILA_NOR (ítem → fila NOR que lo trata, porque el auditor y el informe numeran distinto: ficha EXT-11-03); cada fila NOR del censo tiene que existir y no estar abierta; el censo se achica solo cuando el tracker absorbe un ítem. El tracker se lee con tests/apoyo/tracker.py (zipfile + xml, sin openpyxl: no abre un tercer eje de entorno).</t>
+          <t>e734c23 — EXT-11 (2026-09-21): el cruce como test en tests/test_ext11_cruce_temarios.py: 71 ítems ALTA/CRÍTICA (severidad final si hay veredicto, propuesta si no), 26 cubiertos por fila propia o mención en el tracker y 45 por el censo CUBIERTOS_POR_FILA_NOR (ítem → fila NOR que lo trata, porque el auditor y el informe numeran distinto: ficha EXT-11-03); cada fila NOR del censo tiene que existir y no estar abierta; el censo se achica solo cuando el tracker absorbe un ítem. El tracker se lee con tests/apoyo/tracker.py (zipfile + xml, sin openpyxl: no abre un tercer eje de entorno).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cierre(PF-1), parte 1: PC-03 cerrado en el tracker con el SHA de ext(PF-1)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014UNRGv9HEMshUs5i81aWtA
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -17330,15 +17330,19 @@
       </c>
       <c r="J264" s="6" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K264" s="6" t="inlineStr">
         <is>
-          <t>pendiente — cadena EXT (docs/planes_mejora/07_CADENA_PROMPTS_EXT.md)</t>
-        </is>
-      </c>
-      <c r="L264" s="6" t="n"/>
+          <t>Claude Code (PF-1)</t>
+        </is>
+      </c>
+      <c r="L264" s="6" t="inlineStr">
+        <is>
+          <t>e29b363 (ext(PF-1))</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="5" t="inlineStr">

</xml_diff>

<commit_message>
cierre(PF-6): sellos sobre 6fbe21a y R48-007 cerrado en el tracker con su SHA — 4112 passed, 3 skipped (PyMuPDF sí · ventana Tk sí)
Sólo cambian la línea del sello de docs/trazabilidad.csv y de
docs/indice_formulas.md (fecha, commit y par, medido sobre un checkout
limpio de 6fbe21a) y la fila R48-007 de la hoja Hallazgos: Estado «Cerrado»,
Responsable con la verificación de PF-6 y Commit «6fbe21a».

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GPbDerPmii1YBYoBgAyghi
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -19434,15 +19434,19 @@
       </c>
       <c r="J298" s="6" t="inlineStr">
         <is>
-          <t>Abierto</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K298" s="6" t="inlineStr">
         <is>
-          <t>pendiente — cadena EXT (docs/planes_mejora/07_CADENA_PROMPTS_EXT.md)</t>
-        </is>
-      </c>
-      <c r="L298" s="6" t="n"/>
+          <t>PF-6 (2026-09-21): verificado contra el PDF del Manual de Suelos (Cuadro 4.11 pág. 37 S5 abierta; Cuadro Nº 10.2 pág. 108 «Mínimo 100%»; Cuadro 12.13 pág. 129 «Base Granular CBR 100%»; sin techo en 281 páginas). CBR_MAX_FISICO retirado; queda dominios.CBR_MIN_FISICO. Ficha PF-6-01.</t>
+        </is>
+      </c>
+      <c r="L298" s="6" t="inlineStr">
+        <is>
+          <t>6fbe21a</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="5" t="inlineStr">

</xml_diff>

<commit_message>
docs(tracker): C5-02 queda abierta sin sesión — EXT-6 no migró la forma de `ke_entrada` (revisión tras PF-6)
Medido sobre origin/main d5ff74c: `ke_entrada` sigue con forma float (0.5) y
`ke_entrada_cajon` con forma str. La fila del tracker apuntaba a EXT-6 como
sesión de cierre y EXT-6 no la tocó; la cadena PF («Después de PF-6») pedía
revisarlo y actualizar el estado sin código. Ficha C5-02 con la revisión.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBQxwVdyW3m3cGwxMRY8MW
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -19782,7 +19782,7 @@
       </c>
       <c r="F304" s="6" t="inlineStr">
         <is>
-          <t>EXT-1 (si cabe) · EXT-6</t>
+          <t>EXT-1 (validación, cerrada) · migración de forma pendiente, sin sesión</t>
         </is>
       </c>
       <c r="G304" s="6" t="inlineStr">
@@ -19802,17 +19802,17 @@
       </c>
       <c r="J304" s="6" t="inlineStr">
         <is>
-          <t>Reabierto (EXT-0) → EXT-6</t>
+          <t>Abierto (mitad de forma; sin sesión asignada)</t>
         </is>
       </c>
       <c r="K304" s="6" t="inlineStr">
         <is>
-          <t>Claude Code (EXT-1) → EXT-6</t>
+          <t>Claude Code (EXT-1) → pendiente, sin sesión asignada</t>
         </is>
       </c>
       <c r="L304" s="6" t="inlineStr">
         <is>
-          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. EXT-1 cerró la mitad de validación (ventana, guardia del consumidor, procedencia veraz) y DIFIERE la migración de forma a EXT-6; ficha C5-02 actualizada en decisiones_diferidas.md.</t>
+          <t>9195e8d — EXT-1 (2026-09-20); el cierre con los sellos es el commit siguiente. Tests de aceptación en tests/test_ext1_entradas.py. EXT-1 cerró la mitad de validación (ventana, guardia del consumidor, procedencia veraz) y DIFIERE la migración de forma a EXT-6; ficha C5-02 actualizada en decisiones_diferidas.md. || Revisión 2026-09-22 (tras PF-6): EXT-6 (363091b) NO migró la forma — medido sobre origin/main d5ff74c: `ke_entrada` sigue con forma float y valor 0.5, `ke_entrada_cajon` con forma str, y `M4.ke_declarado` conserva la rama de rótulos vacíos. Queda ABIERTA sin sesión asignada; la ficha C5-02 de decisiones_diferidas.md dice qué haría falta.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cierre(C10/C05/C09/C11/C14): sellos sobre 19bcf5a, tabla de CLAUDE.md y tracker — 4172 passed, 3 skipped (PyMuPDF sí · ventana Tk sí)
Los cuatro documentos generados regenerados sobre un árbol limpio de 19bcf5a
(manifiesto_citas, manifiesto_registro_normativo, trazabilidad.csv con 186
citas, indice_formulas). Tabla de las cuatro configuraciones medida en serie
sobre un git worktree de origin/main en 19bcf5a (collected 4175 en las
cuatro; los 13 tests de documentos generados fallaban en todas hasta este
sellado y se suman a cada passed). Tracker: C5-02, PC-27, PC-32, PC-24,
R48-030, R48-001, PC-31 cerrados; SIS-F-01, SIS-F-13 y NOR-PRO-04 cerrado
parcial con la razón nueva medida. CLAUDE.md: el párrafo del cierre, los
conteos de criterios (77 desde C10, 79 desde C05) y de ventanas reales.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JBQxwVdyW3m3cGwxMRY8MW
</commit_message>
<xml_diff>
--- a/docs/auditorias/matriz_cruzada_auditorias.xlsx
+++ b/docs/auditorias/matriz_cruzada_auditorias.xlsx
@@ -7037,7 +7037,7 @@
       </c>
       <c r="L87" s="6" t="inlineStr">
         <is>
-          <t>4f92508 — cierre C09 (2026-09-22). Sin cambio de estado; la mitad concreto cambia de razon: «M 170M Tablas 1-5 sin transcribir» pasa a «el ejemplar de normas/ no es transcribible» (medido: imagen recompuesta por OCR con digitos equivocados; ver SIS-F-13 y ficha C09-02). Hace falta otro ejemplar. La mitad TMC sigue esperando la implementacion del procedimiento de A796 en M8 (sesion de calculo propia). Veredicto regla 3: sigue CIERRA EN PARTE. || Anterior: 4141fd5 — S19 — RAZON PRECISADA, y la mitad abierta se parte en dos de dificultad distinta, que es lo que faltaba decir. La atribucion sigue corregida (A796/A796M, con A798 para instalacion) y `clases_producto_por_relleno` sigue vacio (verificado: valor=None). (1) La relacion luz/corrugacion de la Tabla 1 de A760 y la Tabla 6 de M 36 SE PUEDE hacer --- las dos fuentes estan en normas/ y S14 dejo comprobado que A760 es legible renderizando su pag. PDF 3 a escala 2.0 --- pero es TRANSCRIPCION DE TABLA, trabajo de la fase de citas y no de esta. (2) El calibre del TMC por altura de cobertura NO se puede hacer en absoluto: ASTM A796/A796M NO ESTA en normas/ (comprobado: las trece fuentes del directorio no la incluyen) y figura en la §15 del plan como ausencia declarada. || S19d — SHA AÑADIDO, y la nota de arriba se lee bien: sin cambio de CODIGO, no sin commit. La razon precisada SI esta versionada --- es la ficha de este ID en la Parte III de docs/decisiones_diferidas.md, que nace en 4141fd5 (verificado: `git show 4141fd5:docs/decisiones_diferidas.md` ya trae las cuatro fichas NOR). Se corrige la celda y NO el verificador: relajar la exigencia de SHA para toda nota que diga «sin cambio de codigo» seria un guardian que se pone verde sobre una FRASE en vez de sobre el hecho, que es el modo de fallo de FACTOR_MURO_TABLA. || 183415b + 9902b3c — I1/I1b — LA MITAD TRANSCRIBIBLE SE CERRO: Tabla 1 de A760 y Table 6 de M 36 transcritas ENTERAS por metodo IMAGEN (ASTM_A760.T1, AASHTO_M36.T6 en src/normativa/tablas.py), con CorrespondenciaDeTablas CORR-TAMANOS-TMC que declara las dos celdas en que difieren (375, 825). VERIFICACION I1b, tres agentes: dos verificador-normativo confirmaron celda a celda (31 filas, 128 X, notas al pie) y el auditor adversarial hallo TRES celdas aritmeticamente anomalas (100-&gt;264, 21in-&gt;500, 750-&gt;2483); el desempate por relectura de digitos a 26-60x en AMBOS PDF dio que lo anomalo esta IMPRESO en las dos ediciones: es propiedad de la fuente, declarada en T_A760_T1.interpretacion.en_contra, NO se reescribe (regla 8). De la verificacion salio ademas la correccion de la Fuente AASHTO_M36: edicion M 36-03 (2007) (la portada; antes decia 2006 sin sosten), paginacion PorCapitulo del rotulo M 36-n, y el hallazgo de que al ejemplar le falta la pagina impresa M 36-5 (PDF 6 en blanco), declarado en su nota. Veredicto regla 3: CIERRA EN PARTE. Sigue Cerrado parcial por la mitad (2): ASTM A796/A796M ausente (FUENTES_AUSENTES, gabinete). || 6ad08be (+ el commit que escribe este SHA, como en S19d) — N1 — LA MITAD (2) CAMBIO DE NATURALEZA, y por eso sigue Cerrado parcial y no Cerrado. ASTM A796/A796M-13 entro en normas/ (pre-N1) y en el registro (N1: fuentes.ASTM_A796, 21 pags, SHA-1 registrado en fuentes.ASTM_A796 (sin transcribirlo aqui: verificar_sesion lee todo hex como commit), texto_extraible=False por capa duplicada, verificacion por IMAGEN). LEIDA ENTERA: la norma NO TABULA el calibre por altura de cobertura -- es una practica: el espesor es la SALIDA de su procedimiento (num. 7 a 10, area de pared requerida con SF = 2, pandeo, costura, FF) elegida de sus Tablas 2 a 35 (cita ASTM_A796.8.1.1.2#SELECCION), y la cobertura minima sale de las ecs. (13)-(16) del num. 11.1 con pisos de 300/600 mm (ASTM_A796.11.1#PISOS); afirmacion negativa SIN_TABLA_CALIBRE_POR_COBERTURA_A796 con las 21 paginas y los 34 titulos de tabla como ambito --. Se transcribieron ENTERAS, por imagen y verificadas celda a celda por tres verificadores, las siete tablas SI de propiedades seccionales de las corrugaciones del catalogo (ASTM_A796.T3, T5, T7, T9, T11, T15, T17), la carga viva por cobertura (6.2.2.1), los limites de FF (10.2, 10.3) y las cargas por eje (11.1). La ATRIBUCION queda verificada en positivo: A796 num. 22.1 nombra a A807/A807M como practica de INSTALACION (ASTM_A796.22.1), y DIS-HR-A807 paso a RESUELTA con la fila de la Fase 8 de la v8 corregida (nota «Corregido (DIS-HR-A807, N1)»). LO QUE SIGUE ABIERTO: la mitad TMC de 'clases_producto_por_relleno' (valor=None, verificado) ya no espera una fuente ni una transcripcion sino la IMPLEMENTACION del procedimiento de A796 en M8 (sesion de calculo propia, con caso patron y con los [A] que el procedimiento pide); la mitad concreto sigue esperando M 170M Tablas 1-5. Veredicto regla 3: CIERRA EN PARTE -- cierra la atribucion y lo transcribible; NO cierra el valor, y la razon de que no cierre cambio de «fuente ausente» a «procedimiento sin implementar».</t>
+          <t>19bcf5a — cierre C09 (2026-09-22), rehecho tras el auditor. Sin cambio de estado. La mitad concreto de 'clases_producto_por_relleno' sigue esperando las clases D-load (M 170M Tablas 1 a 4, recomposiciones OCR ilegibles en este ejemplar; la Tabla 5 esta transcrita en diametros y paredes, no en areas de refuerzo); la mitad TMC sigue esperando la implementacion del procedimiento de A796 en M8. Veredicto regla 3: sigue CIERRA EN PARTE. || Anterior: 4f92508 — cierre C09 (2026-09-22). Sin cambio de estado; la mitad concreto cambia de razon: «M 170M Tablas 1-5 sin transcribir» pasa a «el ejemplar de normas/ no es transcribible» (medido: imagen recompuesta por OCR con digitos equivocados; ver SIS-F-13 y ficha C09-02). Hace falta otro ejemplar. La mitad TMC sigue esperando la implementacion del procedimiento de A796 en M8 (sesion de calculo propia). Veredicto regla 3: sigue CIERRA EN PARTE. || Anterior: 4141fd5 — S19 — RAZON PRECISADA, y la mitad abierta se parte en dos de dificultad distinta, que es lo que faltaba decir. La atribucion sigue corregida (A796/A796M, con A798 para instalacion) y `clases_producto_por_relleno` sigue vacio (verificado: valor=None). (1) La relacion luz/corrugacion de la Tabla 1 de A760 y la Tabla 6 de M 36 SE PUEDE hacer --- las dos fuentes estan en normas/ y S14 dejo comprobado que A760 es legible renderizando su pag. PDF 3 a escala 2.0 --- pero es TRANSCRIPCION DE TABLA, trabajo de la fase de citas y no de esta. (2) El calibre del TMC por altura de cobertura NO se puede hacer en absoluto: ASTM A796/A796M NO ESTA en normas/ (comprobado: las trece fuentes del directorio no la incluyen) y figura en la §15 del plan como ausencia declarada. || S19d — SHA AÑADIDO, y la nota de arriba se lee bien: sin cambio de CODIGO, no sin commit. La razon precisada SI esta versionada --- es la ficha de este ID en la Parte III de docs/decisiones_diferidas.md, que nace en 4141fd5 (verificado: `git show 4141fd5:docs/decisiones_diferidas.md` ya trae las cuatro fichas NOR). Se corrige la celda y NO el verificador: relajar la exigencia de SHA para toda nota que diga «sin cambio de codigo» seria un guardian que se pone verde sobre una FRASE en vez de sobre el hecho, que es el modo de fallo de FACTOR_MURO_TABLA. || 183415b + 9902b3c — I1/I1b — LA MITAD TRANSCRIBIBLE SE CERRO: Tabla 1 de A760 y Table 6 de M 36 transcritas ENTERAS por metodo IMAGEN (ASTM_A760.T1, AASHTO_M36.T6 en src/normativa/tablas.py), con CorrespondenciaDeTablas CORR-TAMANOS-TMC que declara las dos celdas en que difieren (375, 825). VERIFICACION I1b, tres agentes: dos verificador-normativo confirmaron celda a celda (31 filas, 128 X, notas al pie) y el auditor adversarial hallo TRES celdas aritmeticamente anomalas (100-&gt;264, 21in-&gt;500, 750-&gt;2483); el desempate por relectura de digitos a 26-60x en AMBOS PDF dio que lo anomalo esta IMPRESO en las dos ediciones: es propiedad de la fuente, declarada en T_A760_T1.interpretacion.en_contra, NO se reescribe (regla 8). De la verificacion salio ademas la correccion de la Fuente AASHTO_M36: edicion M 36-03 (2007) (la portada; antes decia 2006 sin sosten), paginacion PorCapitulo del rotulo M 36-n, y el hallazgo de que al ejemplar le falta la pagina impresa M 36-5 (PDF 6 en blanco), declarado en su nota. Veredicto regla 3: CIERRA EN PARTE. Sigue Cerrado parcial por la mitad (2): ASTM A796/A796M ausente (FUENTES_AUSENTES, gabinete). || 6ad08be (+ el commit que escribe este SHA, como en S19d) — N1 — LA MITAD (2) CAMBIO DE NATURALEZA, y por eso sigue Cerrado parcial y no Cerrado. ASTM A796/A796M-13 entro en normas/ (pre-N1) y en el registro (N1: fuentes.ASTM_A796, 21 pags, SHA-1 registrado en fuentes.ASTM_A796 (sin transcribirlo aqui: verificar_sesion lee todo hex como commit), texto_extraible=False por capa duplicada, verificacion por IMAGEN). LEIDA ENTERA: la norma NO TABULA el calibre por altura de cobertura -- es una practica: el espesor es la SALIDA de su procedimiento (num. 7 a 10, area de pared requerida con SF = 2, pandeo, costura, FF) elegida de sus Tablas 2 a 35 (cita ASTM_A796.8.1.1.2#SELECCION), y la cobertura minima sale de las ecs. (13)-(16) del num. 11.1 con pisos de 300/600 mm (ASTM_A796.11.1#PISOS); afirmacion negativa SIN_TABLA_CALIBRE_POR_COBERTURA_A796 con las 21 paginas y los 34 titulos de tabla como ambito --. Se transcribieron ENTERAS, por imagen y verificadas celda a celda por tres verificadores, las siete tablas SI de propiedades seccionales de las corrugaciones del catalogo (ASTM_A796.T3, T5, T7, T9, T11, T15, T17), la carga viva por cobertura (6.2.2.1), los limites de FF (10.2, 10.3) y las cargas por eje (11.1). La ATRIBUCION queda verificada en positivo: A796 num. 22.1 nombra a A807/A807M como practica de INSTALACION (ASTM_A796.22.1), y DIS-HR-A807 paso a RESUELTA con la fila de la Fase 8 de la v8 corregida (nota «Corregido (DIS-HR-A807, N1)»). LO QUE SIGUE ABIERTO: la mitad TMC de 'clases_producto_por_relleno' (valor=None, verificado) ya no espera una fuente ni una transcripcion sino la IMPLEMENTACION del procedimiento de A796 en M8 (sesion de calculo propia, con caso patron y con los [A] que el procedimiento pide); la mitad concreto sigue esperando M 170M Tablas 1-5. Veredicto regla 3: CIERRA EN PARTE -- cierra la atribucion y lo transcribible; NO cierra el valor, y la razon de que no cierre cambio de «fuente ausente» a «procedimiento sin implementar».</t>
         </is>
       </c>
     </row>
@@ -9041,7 +9041,7 @@
       </c>
       <c r="L121" s="6" t="inlineStr">
         <is>
-          <t>4f92508 — cierre C09 (2026-09-22). EL ALCANCE ABIERTO DESDE I1b SE CUBRE: tests/apoyo/gui_caras_normativa.py (decimo test de ventana real, test_gui_contrato::test_las_tres_caras_restantes_se_construyen_y_declaran_de_verdad) construye bajo Tk real las caras RANGO (v_max_concreto_eleccion), CATALOGO (D_max_catalogo) y CAMPO (esviaje_max_grados) —clave por cara medida contra el modelo— y recorre `_declarar` con un valor malo (sin rastro: rotulo «No se declaro», nada en caliente, sin procedencia, sin callback) y uno bueno (los cuatro). LO QUE SIGUE ABIERTO es solo el entorno (CI con servidor X virtual), que es infraestructura y no un test; ficha C09-01. Veredicto regla 3: CIERRA EN PARTE (todo el alcance de codigo; el entorno no es de este repositorio). || Anterior: 4141fd5 — S19 cubre la parte que faltaba DENTRO de la frontera declarada, y la frontera no se mueve. NUEVO: `_estado_criterio` ejercitado en sus tres casos (incluido «declarado (corrida)», el que SIS-A-01 dejo invisible); la leyenda de etiquetas contrastada contra `ca.CRITERIOS` en vez de contra una lista copiada; que `_llenar_tabla_criterios` lea el valor por `ca.criterio_efectivo` y no por una regla propia (SIS-A-01 en forma de guardia); y dos guardias de encabezado contra el arbol --- las cuatro pestanas y las cuatro exportaciones (SIS-A-10, que se habia cerrado a mano y no vigilaba nadie), y que el encabezado no vuelva a afirmar que usa el campo validable. MEDIDO: gui/app.py tiene hoy 1182 lineas y ~595 sentencias ejecutables; la suite ejecuta una fraccion pequeña y el resto se lee del AST. SIGUE ABIERTO, y es lo mismo que S17 declaro: el codigo que CONSTRUYE WIDGETS no se ejecuta en la suite, ni el viejo de gui/app.py ni el nuevo de gui/ventana_normativa.py. No es descuido: con un doble de tkinter seria un espejismo. QUE HARIA FALTA: una suite con Tk real bajo servidor X virtual en CI. Es infraestructura, no un test mas. || 183415b + 9902b3c — I1/I1b — EL HUECO NOMBRADO SE CUBRE, MEDIDO: cuarto test de ventana real (test_la_ventana_normativa_se_construye_y_se_cierra_de_verdad + tests/apoyo/gui_smoke_normativa.py): construye la app bajo Tk real, puebla las cuatro pestañas con el CSV de expediente y abre y cierra gui/ventana_normativa.py por el camino del raton — el archivo no se construia NUNCA en la suite. Censo de CLAUDE.md: cuatro tests de ventana, y la tabla de entornos re-medida en I1b. ALCANCE MEDIDO EN I1b (auditor adversarial): el smoke abre la cara TABLA; _pintar_rango, _pintar_catalogo, _pintar_campo y el camino de _declarar siguen sin construirse bajo Tk — declarado en la ficha de decisiones_diferidas. Veredicto regla 3: CIERRA EN PARTE (la ficha de auditoria es mas ancha: _interpretar_valor_declarado, banderas, cli.correr — eso ya lo cubrio S19 dentro de su frontera). Sigue Cerrado parcial: lo abierto es alcance (tres caras) y entorno (CI sin X).</t>
+          <t>19bcf5a — cierre C09, ajustes del auditor adversarial (2026-09-22): tres mutantes vivos muertos —`_pintar_*` en no-op (ahora se afirma un texto que solo pinta cada cara), boton sin `command` (se declara por `boton.invoke()`), validador de rango anulado (se lee `lbl_validacion` tras teclear 9,0)—. Lo abierto sigue siendo solo el entorno (CI con X virtual). Ficha C09-01. || Anterior: 4f92508 — cierre C09 (2026-09-22). EL ALCANCE ABIERTO DESDE I1b SE CUBRE: tests/apoyo/gui_caras_normativa.py (decimo test de ventana real, test_gui_contrato::test_las_tres_caras_restantes_se_construyen_y_declaran_de_verdad) construye bajo Tk real las caras RANGO (v_max_concreto_eleccion), CATALOGO (D_max_catalogo) y CAMPO (esviaje_max_grados) —clave por cara medida contra el modelo— y recorre `_declarar` con un valor malo (sin rastro: rotulo «No se declaro», nada en caliente, sin procedencia, sin callback) y uno bueno (los cuatro). LO QUE SIGUE ABIERTO es solo el entorno (CI con servidor X virtual), que es infraestructura y no un test; ficha C09-01. Veredicto regla 3: CIERRA EN PARTE (todo el alcance de codigo; el entorno no es de este repositorio). || Anterior: 4141fd5 — S19 cubre la parte que faltaba DENTRO de la frontera declarada, y la frontera no se mueve. NUEVO: `_estado_criterio` ejercitado en sus tres casos (incluido «declarado (corrida)», el que SIS-A-01 dejo invisible); la leyenda de etiquetas contrastada contra `ca.CRITERIOS` en vez de contra una lista copiada; que `_llenar_tabla_criterios` lea el valor por `ca.criterio_efectivo` y no por una regla propia (SIS-A-01 en forma de guardia); y dos guardias de encabezado contra el arbol --- las cuatro pestanas y las cuatro exportaciones (SIS-A-10, que se habia cerrado a mano y no vigilaba nadie), y que el encabezado no vuelva a afirmar que usa el campo validable. MEDIDO: gui/app.py tiene hoy 1182 lineas y ~595 sentencias ejecutables; la suite ejecuta una fraccion pequeña y el resto se lee del AST. SIGUE ABIERTO, y es lo mismo que S17 declaro: el codigo que CONSTRUYE WIDGETS no se ejecuta en la suite, ni el viejo de gui/app.py ni el nuevo de gui/ventana_normativa.py. No es descuido: con un doble de tkinter seria un espejismo. QUE HARIA FALTA: una suite con Tk real bajo servidor X virtual en CI. Es infraestructura, no un test mas. || 183415b + 9902b3c — I1/I1b — EL HUECO NOMBRADO SE CUBRE, MEDIDO: cuarto test de ventana real (test_la_ventana_normativa_se_construye_y_se_cierra_de_verdad + tests/apoyo/gui_smoke_normativa.py): construye la app bajo Tk real, puebla las cuatro pestañas con el CSV de expediente y abre y cierra gui/ventana_normativa.py por el camino del raton — el archivo no se construia NUNCA en la suite. Censo de CLAUDE.md: cuatro tests de ventana, y la tabla de entornos re-medida en I1b. ALCANCE MEDIDO EN I1b (auditor adversarial): el smoke abre la cara TABLA; _pintar_rango, _pintar_catalogo, _pintar_campo y el camino de _declarar siguen sin construirse bajo Tk — declarado en la ficha de decisiones_diferidas. Veredicto regla 3: CIERRA EN PARTE (la ficha de auditoria es mas ancha: _interpretar_valor_declarado, banderas, cli.correr — eso ya lo cubrio S19 dentro de su frontera). Sigue Cerrado parcial: lo abierto es alcance (tres caras) y entorno (CI sin X).</t>
         </is>
       </c>
     </row>
@@ -10147,7 +10147,7 @@
       </c>
       <c r="L140" s="6" t="inlineStr">
         <is>
-          <t>4f92508 — cierre C09 (2026-09-22). LA MITAD CONCRETO SE MIDIO Y NO SE PUEDE: las Tablas 1-5 de M 170M (PDF 3-7) renderizadas a 2.5x son una recomposicion OCR con digitos equivocados en la propia imagen (371 por 375, 1390 por 1350, «3tS0», «6tXI»), filas superpuestas (2100/2250) y PDF 8 y 10 en blanco; transcribir de ahi seria inventar (regla 8). La nota de fuentes.AASHTO_M170M lo dice con esas palabras (test_cierre_varios) en vez de prometer «renderizar la pagina y leerla». Queda: la serie del concreto en CP11 sin dorado hasta conseguir otro ejemplar, y M10 (expediente vial). Ficha C09-02. Veredicto regla 3: NO CIERRA el valor y cierra la RAZON (medida, no supuesta). || Anterior: 4141fd5 — RAZON ESTRECHADA DE TRES A DOS. `test_M5_verificaciones.py` consume ya CP-3 por la cadena de produccion entera (catalogo de M2 -&gt; Manning de M3 -&gt; umbral de M5) sin fabricar ningun dorado: todos los numeros salen de CP-2, CP-3 o de la constante [N] V_MIN, de modo que el conflicto n.7 no se toca. CP-3 gana ademas su propia `tolerancia_V` declarada, y test_M3 deja de escribirla a mano. Y LA REGLA DEJA DE VIVIR SOLO EN CLAUDE.md: test_guardias_de_la_suite.test_todo_modulo_de_calculo_consume_su_caso_patron la ejecuta, con la lista de exentos DECLARADA (M2, M8, M10 con la fuente que falta segun la §15; M11 por no corresponderle dorado) y fallando tambien si un exento deja de serlo. SIGUEN SIN CASO PATRON M2, M8 y M10, por falta de fuente externa: A796/A796M no esta en normas/, y para M10 lo que falta no es una norma sino el expediente vial. || PRECISADO EN S19c tras refutar los tests nuevos: la guardia que se escribio para cerrar este hallazgo decidia si un modulo consume su caso patron con `"casos_patron" in texto`, una busqueda de subcadena --- o sea que cometia SIS-F-17 al cerrar SIS-F-13 ---. Fallaba en las dos direcciones: un modulo podia perder el import Y el test y quedar verde mientras sobreviviera la palabra en un comentario, y un exento que solo la mencionara disparaba la alarma contraria. Reescrita por AST; el mutante muere. Y los DOS tests de CP-3 se rehicieron: el primero anunciaba vigilar la tolerancia de umbral y no la vigila (margen 7.3e-06 contra TOL 1e-09), y el segundo decia ejercitar la conclusion del fixture evaluando FUERA de sus condiciones (y/D caia a 0.32 desde el 0.75 que la conclusion fija). El segundo se reescribio sobre la mitad que nadie ejercitaba: la salvedad de MAT-O20 --- «con y/D &lt; 0.056 V2 SI se viola a S = 0.001» --- era una afirmacion escrita y no comprobada, y ahora se comprueba con su frontera por los dos lados. || 183415b + 9902b3c — I1/I1b — FICHA RECONCILIADA CON LA GUARDIA: M8 salio del censo SIN_CASO_PATRON en C7 (CP10_FLOTACION_MARCO) y la ficha de decisiones_diferidas aun lo listaba; quedan M2 y M10, cada uno con su fuente concreta, sin fabricar dorados (conflicto #7 respetado, verificado por el auditor adversarial). EN I1b ademas la razon de M2 en la guardia se actualizo por el propio trabajo de I1: la serie del TMC dejo de faltar (ASTM_A760.T1/AASHTO_M36.T6, paso 150 mm real sobre 900) y siguen faltando las series del concreto (M 170M Tablas 1-5 sin transcribir) y del HDPE (M294 ausente). Veredicto regla 3: CIERRA EN PARTE. Sigue Cerrado parcial. || 0d1e5fa (N2, 2026-09-14) — M2 SALE DE LA LISTA DE EXENTOS, en dos tercios y sin fabricar nada: la traduccion no oficial de AASHTO M 294-11 entro en normas/ y su serie de tamaños nominales (7.2.1, tabla de 7.2.2, `AASHTO_M294_TRAD.T7.2.2`) esta transcrita, de modo que con la del TMC (I1) hay dorado de TABLA para dos de los tres materiales: `CP11_SERIES_NOMINALES` en casos_patron.py y seis tests en test_M2 que contrastan `siguiente_diametro` contra las tablas del registro y no contra la formula (conflicto #7 respetado). El dorado del HDPE acredita lo que la traduccion imprime (sin firma; el original sigue ausente). Lo que sigue abierto: la serie del concreto (M 170M Tablas 1-5 sin transcribir), censada en el propio fixture (`['concreto_reforzado'] is None`, con test), y M10 (expediente vial). Veredicto regla 3: CIERRA EN PARTE. Sigue Cerrado parcial.</t>
+          <t>19bcf5a — cierre C09 REHECHO tras el auditor adversarial (2026-09-22): la primera version decia «PDF 8 y 10 en blanco; hace falta otro ejemplar» y era FALSA para la PDF 10, que es un escaneo real, legible, girado 90 grados (Tabla 5, Clase V). Transcrita por IMAGEN: `AASHTO_M170M.T5` con los 27 diametros (300 a 3600 mm) y las paredes B (300-1200) y C (300-1800), con interpretacion en contra declarada (las Clases I a IV no se pueden contrastar contra este ejemplar: las Tablas 1 a 4 SI son recomposiciones OCR con digitos equivocados en la imagen, 371 por 375, 1390 por 1350). CP11 tiene dorado de TABLA para los TRES materiales y `M2.siguiente_diametro` se contrasta contra la serie del concreto (test_M2, 5 parametrizados mas). La nota de fuentes.AASHTO_M170M dice cuales tablas son OCR y cual es escaneo. Queda: M10 (expediente vial). Ficha C09-02. Veredicto regla 3: CIERRA la mitad concreto de M2; M10 sigue. || Anterior: 4f92508 — cierre C09 (2026-09-22). LA MITAD CONCRETO SE MIDIO Y NO SE PUEDE: las Tablas 1-5 de M 170M (PDF 3-7) renderizadas a 2.5x son una recomposicion OCR con digitos equivocados en la propia imagen (371 por 375, 1390 por 1350, «3tS0», «6tXI»), filas superpuestas (2100/2250) y PDF 8 y 10 en blanco; transcribir de ahi seria inventar (regla 8). La nota de fuentes.AASHTO_M170M lo dice con esas palabras (test_cierre_varios) en vez de prometer «renderizar la pagina y leerla». Queda: la serie del concreto en CP11 sin dorado hasta conseguir otro ejemplar, y M10 (expediente vial). Ficha C09-02. Veredicto regla 3: NO CIERRA el valor y cierra la RAZON (medida, no supuesta). || Anterior: 4141fd5 — RAZON ESTRECHADA DE TRES A DOS. `test_M5_verificaciones.py` consume ya CP-3 por la cadena de produccion entera (catalogo de M2 -&gt; Manning de M3 -&gt; umbral de M5) sin fabricar ningun dorado: todos los numeros salen de CP-2, CP-3 o de la constante [N] V_MIN, de modo que el conflicto n.7 no se toca. CP-3 gana ademas su propia `tolerancia_V` declarada, y test_M3 deja de escribirla a mano. Y LA REGLA DEJA DE VIVIR SOLO EN CLAUDE.md: test_guardias_de_la_suite.test_todo_modulo_de_calculo_consume_su_caso_patron la ejecuta, con la lista de exentos DECLARADA (M2, M8, M10 con la fuente que falta segun la §15; M11 por no corresponderle dorado) y fallando tambien si un exento deja de serlo. SIGUEN SIN CASO PATRON M2, M8 y M10, por falta de fuente externa: A796/A796M no esta en normas/, y para M10 lo que falta no es una norma sino el expediente vial. || PRECISADO EN S19c tras refutar los tests nuevos: la guardia que se escribio para cerrar este hallazgo decidia si un modulo consume su caso patron con `"casos_patron" in texto`, una busqueda de subcadena --- o sea que cometia SIS-F-17 al cerrar SIS-F-13 ---. Fallaba en las dos direcciones: un modulo podia perder el import Y el test y quedar verde mientras sobreviviera la palabra en un comentario, y un exento que solo la mencionara disparaba la alarma contraria. Reescrita por AST; el mutante muere. Y los DOS tests de CP-3 se rehicieron: el primero anunciaba vigilar la tolerancia de umbral y no la vigila (margen 7.3e-06 contra TOL 1e-09), y el segundo decia ejercitar la conclusion del fixture evaluando FUERA de sus condiciones (y/D caia a 0.32 desde el 0.75 que la conclusion fija). El segundo se reescribio sobre la mitad que nadie ejercitaba: la salvedad de MAT-O20 --- «con y/D &lt; 0.056 V2 SI se viola a S = 0.001» --- era una afirmacion escrita y no comprobada, y ahora se comprueba con su frontera por los dos lados. || 183415b + 9902b3c — I1/I1b — FICHA RECONCILIADA CON LA GUARDIA: M8 salio del censo SIN_CASO_PATRON en C7 (CP10_FLOTACION_MARCO) y la ficha de decisiones_diferidas aun lo listaba; quedan M2 y M10, cada uno con su fuente concreta, sin fabricar dorados (conflicto #7 respetado, verificado por el auditor adversarial). EN I1b ademas la razon de M2 en la guardia se actualizo por el propio trabajo de I1: la serie del TMC dejo de faltar (ASTM_A760.T1/AASHTO_M36.T6, paso 150 mm real sobre 900) y siguen faltando las series del concreto (M 170M Tablas 1-5 sin transcribir) y del HDPE (M294 ausente). Veredicto regla 3: CIERRA EN PARTE. Sigue Cerrado parcial. || 0d1e5fa (N2, 2026-09-14) — M2 SALE DE LA LISTA DE EXENTOS, en dos tercios y sin fabricar nada: la traduccion no oficial de AASHTO M 294-11 entro en normas/ y su serie de tamaños nominales (7.2.1, tabla de 7.2.2, `AASHTO_M294_TRAD.T7.2.2`) esta transcrita, de modo que con la del TMC (I1) hay dorado de TABLA para dos de los tres materiales: `CP11_SERIES_NOMINALES` en casos_patron.py y seis tests en test_M2 que contrastan `siguiente_diametro` contra las tablas del registro y no contra la formula (conflicto #7 respetado). El dorado del HDPE acredita lo que la traduccion imprime (sin firma; el original sigue ausente). Lo que sigue abierto: la serie del concreto (M 170M Tablas 1-5 sin transcribir), censada en el propio fixture (`['concreto_reforzado'] is None`, con test), y M10 (expediente vial). Veredicto regla 3: CIERRA EN PARTE. Sigue Cerrado parcial.</t>
         </is>
       </c>
     </row>
@@ -19510,7 +19510,7 @@
       </c>
       <c r="L299" s="6" t="inlineStr">
         <is>
-          <t>4f92508 — cierre C11 (2026-09-22). LA MAGNITUD QUEDA DICHA: dos citas nuevas verificadas contra el PDF (MP glosario pag. impresa 45 / PDF 46 «OBRAS DE ARTE MENORES: … luz libre es menor que 6.00 m (20 ft)»; AASHTO LRFD 9 Art. 1.2 pag. 1-2 / PDF 17 «Bridge—Any structure having an opening not less than 20.0 ft…»), la discrepancia DIS-LUZ-DENOMINACION (ABIERTA, gana AASHTO porque el 4.1.1.5.1 remite a ella) declarada en el paso F2.LUZ (via 2 del canal, test_canal_discrepancias reescrito con el caso real) y en el fundamento, y `luz_m` / la procedencia del paso diciendo que es la ABERTURA libre que el cruce exige de la estructura y NO el ancho del cauce natural; en multicelda, la abertura total (lectura conservadora, declarada como tal: ninguna fuente de normas/ la escribe, ficha C11-01). Tests: test_cierre_varios.py. Veredicto regla 3: CIERRA lo que el hallazgo pedia (nombrar la magnitud y anclarla a las definiciones); la abertura del multicelda queda declarada, no citada.</t>
+          <t>19bcf5a — cierre C11 REHECHO tras el auditor adversarial (2026-09-22), que refuto la primera version («las tres fuentes coinciden», multicelda razonado por cuenta propia): habia dos fuentes en normas/ sin citar. Hoy el registro lleva CINCO citas verificadas contra su pagina: MP glosario pag. 45/PDF 46 («OBRAS DE ARTE MENORES: … luz libre es menor que 6.00 m (20 ft)»), MP Fig. 1.10-a pag. 73/PDF 74 («C = LUZ LIBRE», POR VANO entre pilares: la parte EN CONTRA), AASHTO LRFD 9 Art. 1.2 pag. 1-2/PDF 17 («an opening not less than 20.0 ft»), HDS-5 §1.2 pag. 1.3/PDF 41 («the total width of a multiple barrel crossing» cuenta como puente para el NBIS) y pag. 1.4/PDF 42 (guia hidraulica por barril). DIS-LUZ-DENOMINACION nombra el desacuerdo REAL —por vano contra ancho total; 6.0 m contra 6.096 m— y quien gana en cada cosa: en la magnitud HDS-5 (ancho total del cruce, lectura conservadora), en la cifra el Manual de Hidrologia (6.0 m [N]). Declarada en el paso F2.LUZ (via 2 del canal) y en el fundamento; `luz_m` y la procedencia dicen que es la abertura de la ESTRUCTURA y NO el ancho del cauce. El caso del hallazgo (8 m / 3 x 2.5) sigue siendo PUENTE, ahora con la fuente que lo sostiene. Tests: test_cierre_varios.py. Ficha C11-01. Veredicto regla 3: CIERRA. || Anterior: 4f92508 — cierre C11 (2026-09-22). LA MAGNITUD QUEDA DICHA: dos citas nuevas verificadas contra el PDF (MP glosario pag. impresa 45 / PDF 46 «OBRAS DE ARTE MENORES: … luz libre es menor que 6.00 m (20 ft)»; AASHTO LRFD 9 Art. 1.2 pag. 1-2 / PDF 17 «Bridge—Any structure having an opening not less than 20.0 ft…»), la discrepancia DIS-LUZ-DENOMINACION (ABIERTA, gana AASHTO porque el 4.1.1.5.1 remite a ella) declarada en el paso F2.LUZ (via 2 del canal, test_canal_discrepancias reescrito con el caso real) y en el fundamento, y `luz_m` / la procedencia del paso diciendo que es la ABERTURA libre que el cruce exige de la estructura y NO el ancho del cauce natural; en multicelda, la abertura total (lectura conservadora, declarada como tal: ninguna fuente de normas/ la escribe, ficha C11-01). Tests: test_cierre_varios.py. Veredicto regla 3: CIERRA lo que el hallazgo pedia (nombrar la magnitud y anclarla a las definiciones); la abertura del multicelda queda declarada, no citada.</t>
         </is>
       </c>
     </row>

</xml_diff>